<commit_message>
Provides both the JSON and Excel files
</commit_message>
<xml_diff>
--- a/CCD-Bench/CCD-Bench_Business_V1.xlsx
+++ b/CCD-Bench/CCD-Bench_Business_V1.xlsx
@@ -1,15 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Data Storage\POLIMI\Semester 2\Multidisciplinary Project\LLM Culture Map Project\Code\CCD-Bench\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F9FFF30-F6B8-40C9-B63B-46F9B6C3B39D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519"/>
 </workbook>
 </file>
 
@@ -15409,8 +15415,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -15447,13 +15453,21 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -15491,7 +15505,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -15525,6 +15539,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -15559,9 +15574,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -15734,11 +15750,19 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:N394"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="9.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="187.88671875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="147" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="155.5546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="214.5546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="242.109375" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:14">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -15782,7 +15806,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:14">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>14</v>
       </c>
@@ -15826,7 +15850,7 @@
         <v>4737</v>
       </c>
     </row>
-    <row r="3" spans="1:14">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>14</v>
       </c>
@@ -15870,7 +15894,7 @@
         <v>4738</v>
       </c>
     </row>
-    <row r="4" spans="1:14">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>15</v>
       </c>
@@ -15914,7 +15938,7 @@
         <v>4739</v>
       </c>
     </row>
-    <row r="5" spans="1:14">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>14</v>
       </c>
@@ -15958,7 +15982,7 @@
         <v>4740</v>
       </c>
     </row>
-    <row r="6" spans="1:14">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>16</v>
       </c>
@@ -16002,7 +16026,7 @@
         <v>4741</v>
       </c>
     </row>
-    <row r="7" spans="1:14">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>14</v>
       </c>
@@ -16046,7 +16070,7 @@
         <v>4742</v>
       </c>
     </row>
-    <row r="8" spans="1:14">
+    <row r="8" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>17</v>
       </c>
@@ -16090,7 +16114,7 @@
         <v>4743</v>
       </c>
     </row>
-    <row r="9" spans="1:14">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>14</v>
       </c>
@@ -16134,7 +16158,7 @@
         <v>4744</v>
       </c>
     </row>
-    <row r="10" spans="1:14">
+    <row r="10" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>18</v>
       </c>
@@ -16178,7 +16202,7 @@
         <v>4745</v>
       </c>
     </row>
-    <row r="11" spans="1:14">
+    <row r="11" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>14</v>
       </c>
@@ -16222,7 +16246,7 @@
         <v>4746</v>
       </c>
     </row>
-    <row r="12" spans="1:14">
+    <row r="12" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>14</v>
       </c>
@@ -16266,7 +16290,7 @@
         <v>4747</v>
       </c>
     </row>
-    <row r="13" spans="1:14">
+    <row r="13" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>14</v>
       </c>
@@ -16310,7 +16334,7 @@
         <v>4748</v>
       </c>
     </row>
-    <row r="14" spans="1:14">
+    <row r="14" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>18</v>
       </c>
@@ -16354,7 +16378,7 @@
         <v>4749</v>
       </c>
     </row>
-    <row r="15" spans="1:14">
+    <row r="15" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>19</v>
       </c>
@@ -16398,7 +16422,7 @@
         <v>4750</v>
       </c>
     </row>
-    <row r="16" spans="1:14">
+    <row r="16" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>14</v>
       </c>
@@ -16442,7 +16466,7 @@
         <v>4751</v>
       </c>
     </row>
-    <row r="17" spans="1:14">
+    <row r="17" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>14</v>
       </c>
@@ -16486,7 +16510,7 @@
         <v>4752</v>
       </c>
     </row>
-    <row r="18" spans="1:14">
+    <row r="18" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>18</v>
       </c>
@@ -16530,7 +16554,7 @@
         <v>4753</v>
       </c>
     </row>
-    <row r="19" spans="1:14">
+    <row r="19" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>18</v>
       </c>
@@ -16574,7 +16598,7 @@
         <v>4754</v>
       </c>
     </row>
-    <row r="20" spans="1:14">
+    <row r="20" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>16</v>
       </c>
@@ -16618,7 +16642,7 @@
         <v>4755</v>
       </c>
     </row>
-    <row r="21" spans="1:14">
+    <row r="21" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>14</v>
       </c>
@@ -16662,7 +16686,7 @@
         <v>4756</v>
       </c>
     </row>
-    <row r="22" spans="1:14">
+    <row r="22" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>14</v>
       </c>
@@ -16706,7 +16730,7 @@
         <v>4757</v>
       </c>
     </row>
-    <row r="23" spans="1:14">
+    <row r="23" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>18</v>
       </c>
@@ -16750,7 +16774,7 @@
         <v>4758</v>
       </c>
     </row>
-    <row r="24" spans="1:14">
+    <row r="24" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>18</v>
       </c>
@@ -16794,7 +16818,7 @@
         <v>4759</v>
       </c>
     </row>
-    <row r="25" spans="1:14">
+    <row r="25" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>14</v>
       </c>
@@ -16838,7 +16862,7 @@
         <v>4760</v>
       </c>
     </row>
-    <row r="26" spans="1:14">
+    <row r="26" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>14</v>
       </c>
@@ -16882,7 +16906,7 @@
         <v>4761</v>
       </c>
     </row>
-    <row r="27" spans="1:14">
+    <row r="27" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>15</v>
       </c>
@@ -16926,7 +16950,7 @@
         <v>4762</v>
       </c>
     </row>
-    <row r="28" spans="1:14">
+    <row r="28" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>14</v>
       </c>
@@ -16970,7 +16994,7 @@
         <v>4763</v>
       </c>
     </row>
-    <row r="29" spans="1:14">
+    <row r="29" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>16</v>
       </c>
@@ -17014,7 +17038,7 @@
         <v>4764</v>
       </c>
     </row>
-    <row r="30" spans="1:14">
+    <row r="30" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>14</v>
       </c>
@@ -17058,7 +17082,7 @@
         <v>4765</v>
       </c>
     </row>
-    <row r="31" spans="1:14">
+    <row r="31" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>15</v>
       </c>
@@ -17102,7 +17126,7 @@
         <v>4766</v>
       </c>
     </row>
-    <row r="32" spans="1:14">
+    <row r="32" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>14</v>
       </c>
@@ -17146,7 +17170,7 @@
         <v>4767</v>
       </c>
     </row>
-    <row r="33" spans="1:14">
+    <row r="33" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>20</v>
       </c>
@@ -17190,7 +17214,7 @@
         <v>4768</v>
       </c>
     </row>
-    <row r="34" spans="1:14">
+    <row r="34" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>14</v>
       </c>
@@ -17234,7 +17258,7 @@
         <v>4769</v>
       </c>
     </row>
-    <row r="35" spans="1:14">
+    <row r="35" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>14</v>
       </c>
@@ -17278,7 +17302,7 @@
         <v>4770</v>
       </c>
     </row>
-    <row r="36" spans="1:14">
+    <row r="36" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>14</v>
       </c>
@@ -17322,7 +17346,7 @@
         <v>4771</v>
       </c>
     </row>
-    <row r="37" spans="1:14">
+    <row r="37" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>14</v>
       </c>
@@ -17366,7 +17390,7 @@
         <v>4772</v>
       </c>
     </row>
-    <row r="38" spans="1:14">
+    <row r="38" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>14</v>
       </c>
@@ -17410,7 +17434,7 @@
         <v>4773</v>
       </c>
     </row>
-    <row r="39" spans="1:14">
+    <row r="39" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>14</v>
       </c>
@@ -17454,7 +17478,7 @@
         <v>4774</v>
       </c>
     </row>
-    <row r="40" spans="1:14">
+    <row r="40" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>14</v>
       </c>
@@ -17498,7 +17522,7 @@
         <v>4775</v>
       </c>
     </row>
-    <row r="41" spans="1:14">
+    <row r="41" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>18</v>
       </c>
@@ -17542,7 +17566,7 @@
         <v>4776</v>
       </c>
     </row>
-    <row r="42" spans="1:14">
+    <row r="42" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>20</v>
       </c>
@@ -17586,7 +17610,7 @@
         <v>4777</v>
       </c>
     </row>
-    <row r="43" spans="1:14">
+    <row r="43" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>18</v>
       </c>
@@ -17630,7 +17654,7 @@
         <v>4778</v>
       </c>
     </row>
-    <row r="44" spans="1:14">
+    <row r="44" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>14</v>
       </c>
@@ -17674,7 +17698,7 @@
         <v>4779</v>
       </c>
     </row>
-    <row r="45" spans="1:14">
+    <row r="45" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>14</v>
       </c>
@@ -17718,7 +17742,7 @@
         <v>4780</v>
       </c>
     </row>
-    <row r="46" spans="1:14">
+    <row r="46" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>17</v>
       </c>
@@ -17762,7 +17786,7 @@
         <v>4781</v>
       </c>
     </row>
-    <row r="47" spans="1:14">
+    <row r="47" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>14</v>
       </c>
@@ -17806,7 +17830,7 @@
         <v>4782</v>
       </c>
     </row>
-    <row r="48" spans="1:14">
+    <row r="48" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
         <v>14</v>
       </c>
@@ -17850,7 +17874,7 @@
         <v>4783</v>
       </c>
     </row>
-    <row r="49" spans="1:14">
+    <row r="49" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
         <v>14</v>
       </c>
@@ -17894,7 +17918,7 @@
         <v>4784</v>
       </c>
     </row>
-    <row r="50" spans="1:14">
+    <row r="50" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
         <v>18</v>
       </c>
@@ -17938,7 +17962,7 @@
         <v>4785</v>
       </c>
     </row>
-    <row r="51" spans="1:14">
+    <row r="51" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
         <v>18</v>
       </c>
@@ -17982,7 +18006,7 @@
         <v>4786</v>
       </c>
     </row>
-    <row r="52" spans="1:14">
+    <row r="52" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
         <v>14</v>
       </c>
@@ -18026,7 +18050,7 @@
         <v>4787</v>
       </c>
     </row>
-    <row r="53" spans="1:14">
+    <row r="53" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
         <v>14</v>
       </c>
@@ -18070,7 +18094,7 @@
         <v>4788</v>
       </c>
     </row>
-    <row r="54" spans="1:14">
+    <row r="54" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
         <v>16</v>
       </c>
@@ -18114,7 +18138,7 @@
         <v>4789</v>
       </c>
     </row>
-    <row r="55" spans="1:14">
+    <row r="55" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
         <v>18</v>
       </c>
@@ -18158,7 +18182,7 @@
         <v>4790</v>
       </c>
     </row>
-    <row r="56" spans="1:14">
+    <row r="56" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
         <v>14</v>
       </c>
@@ -18202,7 +18226,7 @@
         <v>4791</v>
       </c>
     </row>
-    <row r="57" spans="1:14">
+    <row r="57" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
         <v>14</v>
       </c>
@@ -18246,7 +18270,7 @@
         <v>4792</v>
       </c>
     </row>
-    <row r="58" spans="1:14">
+    <row r="58" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
         <v>14</v>
       </c>
@@ -18290,7 +18314,7 @@
         <v>4793</v>
       </c>
     </row>
-    <row r="59" spans="1:14">
+    <row r="59" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
         <v>14</v>
       </c>
@@ -18334,7 +18358,7 @@
         <v>4794</v>
       </c>
     </row>
-    <row r="60" spans="1:14">
+    <row r="60" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
         <v>14</v>
       </c>
@@ -18378,7 +18402,7 @@
         <v>4795</v>
       </c>
     </row>
-    <row r="61" spans="1:14">
+    <row r="61" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
         <v>14</v>
       </c>
@@ -18422,7 +18446,7 @@
         <v>4796</v>
       </c>
     </row>
-    <row r="62" spans="1:14">
+    <row r="62" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
         <v>14</v>
       </c>
@@ -18466,7 +18490,7 @@
         <v>4797</v>
       </c>
     </row>
-    <row r="63" spans="1:14">
+    <row r="63" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
         <v>20</v>
       </c>
@@ -18510,7 +18534,7 @@
         <v>4798</v>
       </c>
     </row>
-    <row r="64" spans="1:14">
+    <row r="64" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
         <v>14</v>
       </c>
@@ -18554,7 +18578,7 @@
         <v>4799</v>
       </c>
     </row>
-    <row r="65" spans="1:14">
+    <row r="65" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
         <v>14</v>
       </c>
@@ -18598,7 +18622,7 @@
         <v>4800</v>
       </c>
     </row>
-    <row r="66" spans="1:14">
+    <row r="66" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
         <v>14</v>
       </c>
@@ -18642,7 +18666,7 @@
         <v>4801</v>
       </c>
     </row>
-    <row r="67" spans="1:14">
+    <row r="67" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
         <v>14</v>
       </c>
@@ -18686,7 +18710,7 @@
         <v>4802</v>
       </c>
     </row>
-    <row r="68" spans="1:14">
+    <row r="68" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
         <v>14</v>
       </c>
@@ -18730,7 +18754,7 @@
         <v>4803</v>
       </c>
     </row>
-    <row r="69" spans="1:14">
+    <row r="69" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
         <v>20</v>
       </c>
@@ -18774,7 +18798,7 @@
         <v>4804</v>
       </c>
     </row>
-    <row r="70" spans="1:14">
+    <row r="70" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
         <v>14</v>
       </c>
@@ -18818,7 +18842,7 @@
         <v>4805</v>
       </c>
     </row>
-    <row r="71" spans="1:14">
+    <row r="71" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
         <v>18</v>
       </c>
@@ -18862,7 +18886,7 @@
         <v>4806</v>
       </c>
     </row>
-    <row r="72" spans="1:14">
+    <row r="72" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
         <v>18</v>
       </c>
@@ -18906,7 +18930,7 @@
         <v>4807</v>
       </c>
     </row>
-    <row r="73" spans="1:14">
+    <row r="73" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
         <v>20</v>
       </c>
@@ -18950,7 +18974,7 @@
         <v>4808</v>
       </c>
     </row>
-    <row r="74" spans="1:14">
+    <row r="74" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
         <v>14</v>
       </c>
@@ -18994,7 +19018,7 @@
         <v>4809</v>
       </c>
     </row>
-    <row r="75" spans="1:14">
+    <row r="75" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
         <v>18</v>
       </c>
@@ -19038,7 +19062,7 @@
         <v>4810</v>
       </c>
     </row>
-    <row r="76" spans="1:14">
+    <row r="76" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
         <v>14</v>
       </c>
@@ -19082,7 +19106,7 @@
         <v>4811</v>
       </c>
     </row>
-    <row r="77" spans="1:14">
+    <row r="77" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
         <v>18</v>
       </c>
@@ -19126,7 +19150,7 @@
         <v>4812</v>
       </c>
     </row>
-    <row r="78" spans="1:14">
+    <row r="78" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
         <v>14</v>
       </c>
@@ -19170,7 +19194,7 @@
         <v>4813</v>
       </c>
     </row>
-    <row r="79" spans="1:14">
+    <row r="79" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
         <v>16</v>
       </c>
@@ -19214,7 +19238,7 @@
         <v>4814</v>
       </c>
     </row>
-    <row r="80" spans="1:14">
+    <row r="80" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
         <v>14</v>
       </c>
@@ -19258,7 +19282,7 @@
         <v>4815</v>
       </c>
     </row>
-    <row r="81" spans="1:14">
+    <row r="81" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
         <v>14</v>
       </c>
@@ -19302,7 +19326,7 @@
         <v>4816</v>
       </c>
     </row>
-    <row r="82" spans="1:14">
+    <row r="82" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
         <v>18</v>
       </c>
@@ -19346,7 +19370,7 @@
         <v>4817</v>
       </c>
     </row>
-    <row r="83" spans="1:14">
+    <row r="83" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A83" t="s">
         <v>16</v>
       </c>
@@ -19390,7 +19414,7 @@
         <v>4818</v>
       </c>
     </row>
-    <row r="84" spans="1:14">
+    <row r="84" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
         <v>14</v>
       </c>
@@ -19434,7 +19458,7 @@
         <v>4819</v>
       </c>
     </row>
-    <row r="85" spans="1:14">
+    <row r="85" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A85" t="s">
         <v>14</v>
       </c>
@@ -19478,7 +19502,7 @@
         <v>4820</v>
       </c>
     </row>
-    <row r="86" spans="1:14">
+    <row r="86" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A86" t="s">
         <v>14</v>
       </c>
@@ -19522,7 +19546,7 @@
         <v>4821</v>
       </c>
     </row>
-    <row r="87" spans="1:14">
+    <row r="87" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A87" t="s">
         <v>14</v>
       </c>
@@ -19566,7 +19590,7 @@
         <v>4822</v>
       </c>
     </row>
-    <row r="88" spans="1:14">
+    <row r="88" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A88" t="s">
         <v>14</v>
       </c>
@@ -19610,7 +19634,7 @@
         <v>4823</v>
       </c>
     </row>
-    <row r="89" spans="1:14">
+    <row r="89" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A89" t="s">
         <v>18</v>
       </c>
@@ -19654,7 +19678,7 @@
         <v>4824</v>
       </c>
     </row>
-    <row r="90" spans="1:14">
+    <row r="90" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A90" t="s">
         <v>14</v>
       </c>
@@ -19698,7 +19722,7 @@
         <v>4825</v>
       </c>
     </row>
-    <row r="91" spans="1:14">
+    <row r="91" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A91" t="s">
         <v>14</v>
       </c>
@@ -19742,7 +19766,7 @@
         <v>4826</v>
       </c>
     </row>
-    <row r="92" spans="1:14">
+    <row r="92" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A92" t="s">
         <v>14</v>
       </c>
@@ -19786,7 +19810,7 @@
         <v>4827</v>
       </c>
     </row>
-    <row r="93" spans="1:14">
+    <row r="93" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A93" t="s">
         <v>18</v>
       </c>
@@ -19830,7 +19854,7 @@
         <v>4828</v>
       </c>
     </row>
-    <row r="94" spans="1:14">
+    <row r="94" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A94" t="s">
         <v>14</v>
       </c>
@@ -19874,7 +19898,7 @@
         <v>4829</v>
       </c>
     </row>
-    <row r="95" spans="1:14">
+    <row r="95" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A95" t="s">
         <v>17</v>
       </c>
@@ -19918,7 +19942,7 @@
         <v>4830</v>
       </c>
     </row>
-    <row r="96" spans="1:14">
+    <row r="96" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A96" t="s">
         <v>18</v>
       </c>
@@ -19962,7 +19986,7 @@
         <v>4831</v>
       </c>
     </row>
-    <row r="97" spans="1:14">
+    <row r="97" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A97" t="s">
         <v>14</v>
       </c>
@@ -20006,7 +20030,7 @@
         <v>4832</v>
       </c>
     </row>
-    <row r="98" spans="1:14">
+    <row r="98" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A98" t="s">
         <v>18</v>
       </c>
@@ -20050,7 +20074,7 @@
         <v>4833</v>
       </c>
     </row>
-    <row r="99" spans="1:14">
+    <row r="99" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A99" t="s">
         <v>20</v>
       </c>
@@ -20094,7 +20118,7 @@
         <v>4834</v>
       </c>
     </row>
-    <row r="100" spans="1:14">
+    <row r="100" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A100" t="s">
         <v>14</v>
       </c>
@@ -20138,7 +20162,7 @@
         <v>4835</v>
       </c>
     </row>
-    <row r="101" spans="1:14">
+    <row r="101" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A101" t="s">
         <v>14</v>
       </c>
@@ -20182,7 +20206,7 @@
         <v>4836</v>
       </c>
     </row>
-    <row r="102" spans="1:14">
+    <row r="102" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A102" t="s">
         <v>18</v>
       </c>
@@ -20226,7 +20250,7 @@
         <v>4837</v>
       </c>
     </row>
-    <row r="103" spans="1:14">
+    <row r="103" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A103" t="s">
         <v>14</v>
       </c>
@@ -20270,7 +20294,7 @@
         <v>4838</v>
       </c>
     </row>
-    <row r="104" spans="1:14">
+    <row r="104" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A104" t="s">
         <v>14</v>
       </c>
@@ -20314,7 +20338,7 @@
         <v>4839</v>
       </c>
     </row>
-    <row r="105" spans="1:14">
+    <row r="105" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A105" t="s">
         <v>18</v>
       </c>
@@ -20358,7 +20382,7 @@
         <v>4840</v>
       </c>
     </row>
-    <row r="106" spans="1:14">
+    <row r="106" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A106" t="s">
         <v>18</v>
       </c>
@@ -20402,7 +20426,7 @@
         <v>4841</v>
       </c>
     </row>
-    <row r="107" spans="1:14">
+    <row r="107" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A107" t="s">
         <v>20</v>
       </c>
@@ -20446,7 +20470,7 @@
         <v>4842</v>
       </c>
     </row>
-    <row r="108" spans="1:14">
+    <row r="108" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A108" t="s">
         <v>17</v>
       </c>
@@ -20490,7 +20514,7 @@
         <v>4843</v>
       </c>
     </row>
-    <row r="109" spans="1:14">
+    <row r="109" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A109" t="s">
         <v>14</v>
       </c>
@@ -20534,7 +20558,7 @@
         <v>4844</v>
       </c>
     </row>
-    <row r="110" spans="1:14">
+    <row r="110" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A110" t="s">
         <v>14</v>
       </c>
@@ -20578,7 +20602,7 @@
         <v>4845</v>
       </c>
     </row>
-    <row r="111" spans="1:14">
+    <row r="111" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A111" t="s">
         <v>18</v>
       </c>
@@ -20622,7 +20646,7 @@
         <v>4846</v>
       </c>
     </row>
-    <row r="112" spans="1:14">
+    <row r="112" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A112" t="s">
         <v>14</v>
       </c>
@@ -20666,7 +20690,7 @@
         <v>4847</v>
       </c>
     </row>
-    <row r="113" spans="1:14">
+    <row r="113" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A113" t="s">
         <v>14</v>
       </c>
@@ -20710,7 +20734,7 @@
         <v>4848</v>
       </c>
     </row>
-    <row r="114" spans="1:14">
+    <row r="114" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A114" t="s">
         <v>14</v>
       </c>
@@ -20754,7 +20778,7 @@
         <v>4849</v>
       </c>
     </row>
-    <row r="115" spans="1:14">
+    <row r="115" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A115" t="s">
         <v>14</v>
       </c>
@@ -20798,7 +20822,7 @@
         <v>4850</v>
       </c>
     </row>
-    <row r="116" spans="1:14">
+    <row r="116" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A116" t="s">
         <v>14</v>
       </c>
@@ -20842,7 +20866,7 @@
         <v>4851</v>
       </c>
     </row>
-    <row r="117" spans="1:14">
+    <row r="117" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A117" t="s">
         <v>14</v>
       </c>
@@ -20886,7 +20910,7 @@
         <v>4852</v>
       </c>
     </row>
-    <row r="118" spans="1:14">
+    <row r="118" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A118" t="s">
         <v>18</v>
       </c>
@@ -20930,7 +20954,7 @@
         <v>4853</v>
       </c>
     </row>
-    <row r="119" spans="1:14">
+    <row r="119" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A119" t="s">
         <v>14</v>
       </c>
@@ -20974,7 +20998,7 @@
         <v>4854</v>
       </c>
     </row>
-    <row r="120" spans="1:14">
+    <row r="120" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A120" t="s">
         <v>18</v>
       </c>
@@ -21018,7 +21042,7 @@
         <v>4855</v>
       </c>
     </row>
-    <row r="121" spans="1:14">
+    <row r="121" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A121" t="s">
         <v>14</v>
       </c>
@@ -21062,7 +21086,7 @@
         <v>4856</v>
       </c>
     </row>
-    <row r="122" spans="1:14">
+    <row r="122" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A122" t="s">
         <v>18</v>
       </c>
@@ -21106,7 +21130,7 @@
         <v>4857</v>
       </c>
     </row>
-    <row r="123" spans="1:14">
+    <row r="123" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A123" t="s">
         <v>20</v>
       </c>
@@ -21150,7 +21174,7 @@
         <v>4858</v>
       </c>
     </row>
-    <row r="124" spans="1:14">
+    <row r="124" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A124" t="s">
         <v>18</v>
       </c>
@@ -21194,7 +21218,7 @@
         <v>4859</v>
       </c>
     </row>
-    <row r="125" spans="1:14">
+    <row r="125" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A125" t="s">
         <v>14</v>
       </c>
@@ -21238,7 +21262,7 @@
         <v>4860</v>
       </c>
     </row>
-    <row r="126" spans="1:14">
+    <row r="126" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A126" t="s">
         <v>14</v>
       </c>
@@ -21282,7 +21306,7 @@
         <v>4861</v>
       </c>
     </row>
-    <row r="127" spans="1:14">
+    <row r="127" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A127" t="s">
         <v>18</v>
       </c>
@@ -21326,7 +21350,7 @@
         <v>4862</v>
       </c>
     </row>
-    <row r="128" spans="1:14">
+    <row r="128" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A128" t="s">
         <v>14</v>
       </c>
@@ -21370,7 +21394,7 @@
         <v>4863</v>
       </c>
     </row>
-    <row r="129" spans="1:14">
+    <row r="129" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A129" t="s">
         <v>14</v>
       </c>
@@ -21414,7 +21438,7 @@
         <v>4864</v>
       </c>
     </row>
-    <row r="130" spans="1:14">
+    <row r="130" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A130" t="s">
         <v>14</v>
       </c>
@@ -21458,7 +21482,7 @@
         <v>4865</v>
       </c>
     </row>
-    <row r="131" spans="1:14">
+    <row r="131" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A131" t="s">
         <v>14</v>
       </c>
@@ -21502,7 +21526,7 @@
         <v>4866</v>
       </c>
     </row>
-    <row r="132" spans="1:14">
+    <row r="132" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A132" t="s">
         <v>14</v>
       </c>
@@ -21546,7 +21570,7 @@
         <v>4867</v>
       </c>
     </row>
-    <row r="133" spans="1:14">
+    <row r="133" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A133" t="s">
         <v>14</v>
       </c>
@@ -21590,7 +21614,7 @@
         <v>4868</v>
       </c>
     </row>
-    <row r="134" spans="1:14">
+    <row r="134" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A134" t="s">
         <v>18</v>
       </c>
@@ -21634,7 +21658,7 @@
         <v>4869</v>
       </c>
     </row>
-    <row r="135" spans="1:14">
+    <row r="135" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A135" t="s">
         <v>18</v>
       </c>
@@ -21678,7 +21702,7 @@
         <v>4870</v>
       </c>
     </row>
-    <row r="136" spans="1:14">
+    <row r="136" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A136" t="s">
         <v>14</v>
       </c>
@@ -21722,7 +21746,7 @@
         <v>4871</v>
       </c>
     </row>
-    <row r="137" spans="1:14">
+    <row r="137" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A137" t="s">
         <v>14</v>
       </c>
@@ -21766,7 +21790,7 @@
         <v>4872</v>
       </c>
     </row>
-    <row r="138" spans="1:14">
+    <row r="138" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A138" t="s">
         <v>14</v>
       </c>
@@ -21810,7 +21834,7 @@
         <v>4873</v>
       </c>
     </row>
-    <row r="139" spans="1:14">
+    <row r="139" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A139" t="s">
         <v>18</v>
       </c>
@@ -21854,7 +21878,7 @@
         <v>4874</v>
       </c>
     </row>
-    <row r="140" spans="1:14">
+    <row r="140" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A140" t="s">
         <v>14</v>
       </c>
@@ -21898,7 +21922,7 @@
         <v>4875</v>
       </c>
     </row>
-    <row r="141" spans="1:14">
+    <row r="141" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A141" t="s">
         <v>14</v>
       </c>
@@ -21942,7 +21966,7 @@
         <v>4876</v>
       </c>
     </row>
-    <row r="142" spans="1:14">
+    <row r="142" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A142" t="s">
         <v>14</v>
       </c>
@@ -21986,7 +22010,7 @@
         <v>4877</v>
       </c>
     </row>
-    <row r="143" spans="1:14">
+    <row r="143" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A143" t="s">
         <v>14</v>
       </c>
@@ -22030,7 +22054,7 @@
         <v>4878</v>
       </c>
     </row>
-    <row r="144" spans="1:14">
+    <row r="144" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A144" t="s">
         <v>17</v>
       </c>
@@ -22074,7 +22098,7 @@
         <v>4879</v>
       </c>
     </row>
-    <row r="145" spans="1:14">
+    <row r="145" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A145" t="s">
         <v>18</v>
       </c>
@@ -22118,7 +22142,7 @@
         <v>4880</v>
       </c>
     </row>
-    <row r="146" spans="1:14">
+    <row r="146" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A146" t="s">
         <v>14</v>
       </c>
@@ -22162,7 +22186,7 @@
         <v>4881</v>
       </c>
     </row>
-    <row r="147" spans="1:14">
+    <row r="147" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A147" t="s">
         <v>14</v>
       </c>
@@ -22206,7 +22230,7 @@
         <v>4882</v>
       </c>
     </row>
-    <row r="148" spans="1:14">
+    <row r="148" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A148" t="s">
         <v>15</v>
       </c>
@@ -22250,7 +22274,7 @@
         <v>4883</v>
       </c>
     </row>
-    <row r="149" spans="1:14">
+    <row r="149" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A149" t="s">
         <v>18</v>
       </c>
@@ -22294,7 +22318,7 @@
         <v>4884</v>
       </c>
     </row>
-    <row r="150" spans="1:14">
+    <row r="150" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A150" t="s">
         <v>14</v>
       </c>
@@ -22338,7 +22362,7 @@
         <v>4885</v>
       </c>
     </row>
-    <row r="151" spans="1:14">
+    <row r="151" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A151" t="s">
         <v>18</v>
       </c>
@@ -22382,7 +22406,7 @@
         <v>4886</v>
       </c>
     </row>
-    <row r="152" spans="1:14">
+    <row r="152" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A152" t="s">
         <v>14</v>
       </c>
@@ -22426,7 +22450,7 @@
         <v>4887</v>
       </c>
     </row>
-    <row r="153" spans="1:14">
+    <row r="153" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A153" t="s">
         <v>14</v>
       </c>
@@ -22470,7 +22494,7 @@
         <v>4888</v>
       </c>
     </row>
-    <row r="154" spans="1:14">
+    <row r="154" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A154" t="s">
         <v>18</v>
       </c>
@@ -22514,7 +22538,7 @@
         <v>4889</v>
       </c>
     </row>
-    <row r="155" spans="1:14">
+    <row r="155" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A155" t="s">
         <v>20</v>
       </c>
@@ -22558,7 +22582,7 @@
         <v>4890</v>
       </c>
     </row>
-    <row r="156" spans="1:14">
+    <row r="156" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A156" t="s">
         <v>18</v>
       </c>
@@ -22602,7 +22626,7 @@
         <v>4891</v>
       </c>
     </row>
-    <row r="157" spans="1:14">
+    <row r="157" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A157" t="s">
         <v>14</v>
       </c>
@@ -22646,7 +22670,7 @@
         <v>4892</v>
       </c>
     </row>
-    <row r="158" spans="1:14">
+    <row r="158" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A158" t="s">
         <v>20</v>
       </c>
@@ -22690,7 +22714,7 @@
         <v>4893</v>
       </c>
     </row>
-    <row r="159" spans="1:14">
+    <row r="159" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A159" t="s">
         <v>20</v>
       </c>
@@ -22734,7 +22758,7 @@
         <v>4894</v>
       </c>
     </row>
-    <row r="160" spans="1:14">
+    <row r="160" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A160" t="s">
         <v>14</v>
       </c>
@@ -22778,7 +22802,7 @@
         <v>4895</v>
       </c>
     </row>
-    <row r="161" spans="1:14">
+    <row r="161" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A161" t="s">
         <v>14</v>
       </c>
@@ -22822,7 +22846,7 @@
         <v>4896</v>
       </c>
     </row>
-    <row r="162" spans="1:14">
+    <row r="162" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A162" t="s">
         <v>14</v>
       </c>
@@ -22866,7 +22890,7 @@
         <v>4897</v>
       </c>
     </row>
-    <row r="163" spans="1:14">
+    <row r="163" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A163" t="s">
         <v>18</v>
       </c>
@@ -22910,7 +22934,7 @@
         <v>4898</v>
       </c>
     </row>
-    <row r="164" spans="1:14">
+    <row r="164" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A164" t="s">
         <v>18</v>
       </c>
@@ -22954,7 +22978,7 @@
         <v>4899</v>
       </c>
     </row>
-    <row r="165" spans="1:14">
+    <row r="165" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A165" t="s">
         <v>19</v>
       </c>
@@ -22998,7 +23022,7 @@
         <v>4900</v>
       </c>
     </row>
-    <row r="166" spans="1:14">
+    <row r="166" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A166" t="s">
         <v>14</v>
       </c>
@@ -23042,7 +23066,7 @@
         <v>4901</v>
       </c>
     </row>
-    <row r="167" spans="1:14">
+    <row r="167" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A167" t="s">
         <v>16</v>
       </c>
@@ -23086,7 +23110,7 @@
         <v>4902</v>
       </c>
     </row>
-    <row r="168" spans="1:14">
+    <row r="168" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A168" t="s">
         <v>14</v>
       </c>
@@ -23130,7 +23154,7 @@
         <v>4903</v>
       </c>
     </row>
-    <row r="169" spans="1:14">
+    <row r="169" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A169" t="s">
         <v>14</v>
       </c>
@@ -23174,7 +23198,7 @@
         <v>4904</v>
       </c>
     </row>
-    <row r="170" spans="1:14">
+    <row r="170" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A170" t="s">
         <v>14</v>
       </c>
@@ -23218,7 +23242,7 @@
         <v>4905</v>
       </c>
     </row>
-    <row r="171" spans="1:14">
+    <row r="171" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A171" t="s">
         <v>18</v>
       </c>
@@ -23262,7 +23286,7 @@
         <v>4906</v>
       </c>
     </row>
-    <row r="172" spans="1:14">
+    <row r="172" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A172" t="s">
         <v>18</v>
       </c>
@@ -23306,7 +23330,7 @@
         <v>4907</v>
       </c>
     </row>
-    <row r="173" spans="1:14">
+    <row r="173" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A173" t="s">
         <v>14</v>
       </c>
@@ -23350,7 +23374,7 @@
         <v>4908</v>
       </c>
     </row>
-    <row r="174" spans="1:14">
+    <row r="174" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A174" t="s">
         <v>14</v>
       </c>
@@ -23394,7 +23418,7 @@
         <v>4909</v>
       </c>
     </row>
-    <row r="175" spans="1:14">
+    <row r="175" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A175" t="s">
         <v>14</v>
       </c>
@@ -23438,7 +23462,7 @@
         <v>4910</v>
       </c>
     </row>
-    <row r="176" spans="1:14">
+    <row r="176" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A176" t="s">
         <v>14</v>
       </c>
@@ -23482,7 +23506,7 @@
         <v>4911</v>
       </c>
     </row>
-    <row r="177" spans="1:14">
+    <row r="177" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A177" t="s">
         <v>14</v>
       </c>
@@ -23526,7 +23550,7 @@
         <v>4912</v>
       </c>
     </row>
-    <row r="178" spans="1:14">
+    <row r="178" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A178" t="s">
         <v>14</v>
       </c>
@@ -23570,7 +23594,7 @@
         <v>4913</v>
       </c>
     </row>
-    <row r="179" spans="1:14">
+    <row r="179" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A179" t="s">
         <v>14</v>
       </c>
@@ -23614,7 +23638,7 @@
         <v>4914</v>
       </c>
     </row>
-    <row r="180" spans="1:14">
+    <row r="180" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A180" t="s">
         <v>14</v>
       </c>
@@ -23658,7 +23682,7 @@
         <v>4915</v>
       </c>
     </row>
-    <row r="181" spans="1:14">
+    <row r="181" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A181" t="s">
         <v>19</v>
       </c>
@@ -23702,7 +23726,7 @@
         <v>4916</v>
       </c>
     </row>
-    <row r="182" spans="1:14">
+    <row r="182" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A182" t="s">
         <v>14</v>
       </c>
@@ -23746,7 +23770,7 @@
         <v>4917</v>
       </c>
     </row>
-    <row r="183" spans="1:14">
+    <row r="183" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A183" t="s">
         <v>18</v>
       </c>
@@ -23790,7 +23814,7 @@
         <v>4918</v>
       </c>
     </row>
-    <row r="184" spans="1:14">
+    <row r="184" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A184" t="s">
         <v>14</v>
       </c>
@@ -23834,7 +23858,7 @@
         <v>4919</v>
       </c>
     </row>
-    <row r="185" spans="1:14">
+    <row r="185" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A185" t="s">
         <v>14</v>
       </c>
@@ -23878,7 +23902,7 @@
         <v>4920</v>
       </c>
     </row>
-    <row r="186" spans="1:14">
+    <row r="186" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A186" t="s">
         <v>15</v>
       </c>
@@ -23922,7 +23946,7 @@
         <v>4921</v>
       </c>
     </row>
-    <row r="187" spans="1:14">
+    <row r="187" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A187" t="s">
         <v>16</v>
       </c>
@@ -23966,7 +23990,7 @@
         <v>4922</v>
       </c>
     </row>
-    <row r="188" spans="1:14">
+    <row r="188" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A188" t="s">
         <v>18</v>
       </c>
@@ -24010,7 +24034,7 @@
         <v>4923</v>
       </c>
     </row>
-    <row r="189" spans="1:14">
+    <row r="189" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A189" t="s">
         <v>19</v>
       </c>
@@ -24054,7 +24078,7 @@
         <v>4924</v>
       </c>
     </row>
-    <row r="190" spans="1:14">
+    <row r="190" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A190" t="s">
         <v>14</v>
       </c>
@@ -24098,7 +24122,7 @@
         <v>4925</v>
       </c>
     </row>
-    <row r="191" spans="1:14">
+    <row r="191" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A191" t="s">
         <v>14</v>
       </c>
@@ -24142,7 +24166,7 @@
         <v>4926</v>
       </c>
     </row>
-    <row r="192" spans="1:14">
+    <row r="192" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A192" t="s">
         <v>18</v>
       </c>
@@ -24186,7 +24210,7 @@
         <v>4927</v>
       </c>
     </row>
-    <row r="193" spans="1:14">
+    <row r="193" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A193" t="s">
         <v>14</v>
       </c>
@@ -24230,7 +24254,7 @@
         <v>4928</v>
       </c>
     </row>
-    <row r="194" spans="1:14">
+    <row r="194" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A194" t="s">
         <v>20</v>
       </c>
@@ -24274,7 +24298,7 @@
         <v>4929</v>
       </c>
     </row>
-    <row r="195" spans="1:14">
+    <row r="195" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A195" t="s">
         <v>14</v>
       </c>
@@ -24318,7 +24342,7 @@
         <v>4930</v>
       </c>
     </row>
-    <row r="196" spans="1:14">
+    <row r="196" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A196" t="s">
         <v>16</v>
       </c>
@@ -24362,7 +24386,7 @@
         <v>4931</v>
       </c>
     </row>
-    <row r="197" spans="1:14">
+    <row r="197" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A197" t="s">
         <v>14</v>
       </c>
@@ -24406,7 +24430,7 @@
         <v>4932</v>
       </c>
     </row>
-    <row r="198" spans="1:14">
+    <row r="198" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A198" t="s">
         <v>15</v>
       </c>
@@ -24450,7 +24474,7 @@
         <v>4933</v>
       </c>
     </row>
-    <row r="199" spans="1:14">
+    <row r="199" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A199" t="s">
         <v>14</v>
       </c>
@@ -24494,7 +24518,7 @@
         <v>4934</v>
       </c>
     </row>
-    <row r="200" spans="1:14">
+    <row r="200" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A200" t="s">
         <v>14</v>
       </c>
@@ -24538,7 +24562,7 @@
         <v>4935</v>
       </c>
     </row>
-    <row r="201" spans="1:14">
+    <row r="201" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A201" t="s">
         <v>14</v>
       </c>
@@ -24582,7 +24606,7 @@
         <v>4936</v>
       </c>
     </row>
-    <row r="202" spans="1:14">
+    <row r="202" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A202" t="s">
         <v>17</v>
       </c>
@@ -24626,7 +24650,7 @@
         <v>4937</v>
       </c>
     </row>
-    <row r="203" spans="1:14">
+    <row r="203" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A203" t="s">
         <v>14</v>
       </c>
@@ -24670,7 +24694,7 @@
         <v>4938</v>
       </c>
     </row>
-    <row r="204" spans="1:14">
+    <row r="204" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A204" t="s">
         <v>14</v>
       </c>
@@ -24714,7 +24738,7 @@
         <v>4939</v>
       </c>
     </row>
-    <row r="205" spans="1:14">
+    <row r="205" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A205" t="s">
         <v>18</v>
       </c>
@@ -24758,7 +24782,7 @@
         <v>4940</v>
       </c>
     </row>
-    <row r="206" spans="1:14">
+    <row r="206" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A206" t="s">
         <v>14</v>
       </c>
@@ -24802,7 +24826,7 @@
         <v>4941</v>
       </c>
     </row>
-    <row r="207" spans="1:14">
+    <row r="207" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A207" t="s">
         <v>14</v>
       </c>
@@ -24846,7 +24870,7 @@
         <v>4942</v>
       </c>
     </row>
-    <row r="208" spans="1:14">
+    <row r="208" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A208" t="s">
         <v>14</v>
       </c>
@@ -24890,7 +24914,7 @@
         <v>4943</v>
       </c>
     </row>
-    <row r="209" spans="1:14">
+    <row r="209" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A209" t="s">
         <v>14</v>
       </c>
@@ -24934,7 +24958,7 @@
         <v>4944</v>
       </c>
     </row>
-    <row r="210" spans="1:14">
+    <row r="210" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A210" t="s">
         <v>14</v>
       </c>
@@ -24978,7 +25002,7 @@
         <v>4945</v>
       </c>
     </row>
-    <row r="211" spans="1:14">
+    <row r="211" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A211" t="s">
         <v>14</v>
       </c>
@@ -25022,7 +25046,7 @@
         <v>4946</v>
       </c>
     </row>
-    <row r="212" spans="1:14">
+    <row r="212" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A212" t="s">
         <v>16</v>
       </c>
@@ -25066,7 +25090,7 @@
         <v>4947</v>
       </c>
     </row>
-    <row r="213" spans="1:14">
+    <row r="213" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A213" t="s">
         <v>20</v>
       </c>
@@ -25110,7 +25134,7 @@
         <v>4948</v>
       </c>
     </row>
-    <row r="214" spans="1:14">
+    <row r="214" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A214" t="s">
         <v>14</v>
       </c>
@@ -25154,7 +25178,7 @@
         <v>4949</v>
       </c>
     </row>
-    <row r="215" spans="1:14">
+    <row r="215" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A215" t="s">
         <v>15</v>
       </c>
@@ -25198,7 +25222,7 @@
         <v>4950</v>
       </c>
     </row>
-    <row r="216" spans="1:14">
+    <row r="216" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A216" t="s">
         <v>20</v>
       </c>
@@ -25242,7 +25266,7 @@
         <v>4951</v>
       </c>
     </row>
-    <row r="217" spans="1:14">
+    <row r="217" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A217" t="s">
         <v>14</v>
       </c>
@@ -25286,7 +25310,7 @@
         <v>4952</v>
       </c>
     </row>
-    <row r="218" spans="1:14">
+    <row r="218" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A218" t="s">
         <v>14</v>
       </c>
@@ -25330,7 +25354,7 @@
         <v>4953</v>
       </c>
     </row>
-    <row r="219" spans="1:14">
+    <row r="219" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A219" t="s">
         <v>18</v>
       </c>
@@ -25374,7 +25398,7 @@
         <v>4954</v>
       </c>
     </row>
-    <row r="220" spans="1:14">
+    <row r="220" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A220" t="s">
         <v>14</v>
       </c>
@@ -25418,7 +25442,7 @@
         <v>4955</v>
       </c>
     </row>
-    <row r="221" spans="1:14">
+    <row r="221" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A221" t="s">
         <v>14</v>
       </c>
@@ -25462,7 +25486,7 @@
         <v>4956</v>
       </c>
     </row>
-    <row r="222" spans="1:14">
+    <row r="222" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A222" t="s">
         <v>14</v>
       </c>
@@ -25506,7 +25530,7 @@
         <v>4957</v>
       </c>
     </row>
-    <row r="223" spans="1:14">
+    <row r="223" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A223" t="s">
         <v>14</v>
       </c>
@@ -25550,7 +25574,7 @@
         <v>4958</v>
       </c>
     </row>
-    <row r="224" spans="1:14">
+    <row r="224" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A224" t="s">
         <v>18</v>
       </c>
@@ -25594,7 +25618,7 @@
         <v>4959</v>
       </c>
     </row>
-    <row r="225" spans="1:14">
+    <row r="225" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A225" t="s">
         <v>14</v>
       </c>
@@ -25638,7 +25662,7 @@
         <v>4960</v>
       </c>
     </row>
-    <row r="226" spans="1:14">
+    <row r="226" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A226" t="s">
         <v>18</v>
       </c>
@@ -25682,7 +25706,7 @@
         <v>4961</v>
       </c>
     </row>
-    <row r="227" spans="1:14">
+    <row r="227" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A227" t="s">
         <v>18</v>
       </c>
@@ -25726,7 +25750,7 @@
         <v>4962</v>
       </c>
     </row>
-    <row r="228" spans="1:14">
+    <row r="228" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A228" t="s">
         <v>14</v>
       </c>
@@ -25770,7 +25794,7 @@
         <v>4963</v>
       </c>
     </row>
-    <row r="229" spans="1:14">
+    <row r="229" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A229" t="s">
         <v>14</v>
       </c>
@@ -25814,7 +25838,7 @@
         <v>4964</v>
       </c>
     </row>
-    <row r="230" spans="1:14">
+    <row r="230" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A230" t="s">
         <v>16</v>
       </c>
@@ -25858,7 +25882,7 @@
         <v>4965</v>
       </c>
     </row>
-    <row r="231" spans="1:14">
+    <row r="231" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A231" t="s">
         <v>14</v>
       </c>
@@ -25902,7 +25926,7 @@
         <v>4966</v>
       </c>
     </row>
-    <row r="232" spans="1:14">
+    <row r="232" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A232" t="s">
         <v>14</v>
       </c>
@@ -25946,7 +25970,7 @@
         <v>4967</v>
       </c>
     </row>
-    <row r="233" spans="1:14">
+    <row r="233" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A233" t="s">
         <v>14</v>
       </c>
@@ -25990,7 +26014,7 @@
         <v>4968</v>
       </c>
     </row>
-    <row r="234" spans="1:14">
+    <row r="234" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A234" t="s">
         <v>14</v>
       </c>
@@ -26034,7 +26058,7 @@
         <v>4969</v>
       </c>
     </row>
-    <row r="235" spans="1:14">
+    <row r="235" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A235" t="s">
         <v>14</v>
       </c>
@@ -26078,7 +26102,7 @@
         <v>4970</v>
       </c>
     </row>
-    <row r="236" spans="1:14">
+    <row r="236" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A236" t="s">
         <v>20</v>
       </c>
@@ -26122,7 +26146,7 @@
         <v>4971</v>
       </c>
     </row>
-    <row r="237" spans="1:14">
+    <row r="237" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A237" t="s">
         <v>14</v>
       </c>
@@ -26166,7 +26190,7 @@
         <v>4972</v>
       </c>
     </row>
-    <row r="238" spans="1:14">
+    <row r="238" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A238" t="s">
         <v>14</v>
       </c>
@@ -26210,7 +26234,7 @@
         <v>4973</v>
       </c>
     </row>
-    <row r="239" spans="1:14">
+    <row r="239" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A239" t="s">
         <v>18</v>
       </c>
@@ -26254,7 +26278,7 @@
         <v>4974</v>
       </c>
     </row>
-    <row r="240" spans="1:14">
+    <row r="240" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A240" t="s">
         <v>14</v>
       </c>
@@ -26298,7 +26322,7 @@
         <v>4975</v>
       </c>
     </row>
-    <row r="241" spans="1:14">
+    <row r="241" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A241" t="s">
         <v>19</v>
       </c>
@@ -26342,7 +26366,7 @@
         <v>4976</v>
       </c>
     </row>
-    <row r="242" spans="1:14">
+    <row r="242" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A242" t="s">
         <v>14</v>
       </c>
@@ -26386,7 +26410,7 @@
         <v>4977</v>
       </c>
     </row>
-    <row r="243" spans="1:14">
+    <row r="243" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A243" t="s">
         <v>14</v>
       </c>
@@ -26430,7 +26454,7 @@
         <v>4978</v>
       </c>
     </row>
-    <row r="244" spans="1:14">
+    <row r="244" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A244" t="s">
         <v>14</v>
       </c>
@@ -26474,7 +26498,7 @@
         <v>4979</v>
       </c>
     </row>
-    <row r="245" spans="1:14">
+    <row r="245" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A245" t="s">
         <v>18</v>
       </c>
@@ -26518,7 +26542,7 @@
         <v>4980</v>
       </c>
     </row>
-    <row r="246" spans="1:14">
+    <row r="246" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A246" t="s">
         <v>14</v>
       </c>
@@ -26562,7 +26586,7 @@
         <v>4981</v>
       </c>
     </row>
-    <row r="247" spans="1:14">
+    <row r="247" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A247" t="s">
         <v>15</v>
       </c>
@@ -26606,7 +26630,7 @@
         <v>4982</v>
       </c>
     </row>
-    <row r="248" spans="1:14">
+    <row r="248" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A248" t="s">
         <v>18</v>
       </c>
@@ -26650,7 +26674,7 @@
         <v>4983</v>
       </c>
     </row>
-    <row r="249" spans="1:14">
+    <row r="249" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A249" t="s">
         <v>20</v>
       </c>
@@ -26694,7 +26718,7 @@
         <v>4984</v>
       </c>
     </row>
-    <row r="250" spans="1:14">
+    <row r="250" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A250" t="s">
         <v>18</v>
       </c>
@@ -26738,7 +26762,7 @@
         <v>4985</v>
       </c>
     </row>
-    <row r="251" spans="1:14">
+    <row r="251" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A251" t="s">
         <v>14</v>
       </c>
@@ -26782,7 +26806,7 @@
         <v>4986</v>
       </c>
     </row>
-    <row r="252" spans="1:14">
+    <row r="252" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A252" t="s">
         <v>14</v>
       </c>
@@ -26826,7 +26850,7 @@
         <v>4987</v>
       </c>
     </row>
-    <row r="253" spans="1:14">
+    <row r="253" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A253" t="s">
         <v>17</v>
       </c>
@@ -26870,7 +26894,7 @@
         <v>4988</v>
       </c>
     </row>
-    <row r="254" spans="1:14">
+    <row r="254" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A254" t="s">
         <v>20</v>
       </c>
@@ -26914,7 +26938,7 @@
         <v>4989</v>
       </c>
     </row>
-    <row r="255" spans="1:14">
+    <row r="255" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A255" t="s">
         <v>14</v>
       </c>
@@ -26958,7 +26982,7 @@
         <v>4990</v>
       </c>
     </row>
-    <row r="256" spans="1:14">
+    <row r="256" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A256" t="s">
         <v>14</v>
       </c>
@@ -27002,7 +27026,7 @@
         <v>4991</v>
       </c>
     </row>
-    <row r="257" spans="1:14">
+    <row r="257" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A257" t="s">
         <v>14</v>
       </c>
@@ -27046,7 +27070,7 @@
         <v>4992</v>
       </c>
     </row>
-    <row r="258" spans="1:14">
+    <row r="258" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A258" t="s">
         <v>14</v>
       </c>
@@ -27090,7 +27114,7 @@
         <v>4993</v>
       </c>
     </row>
-    <row r="259" spans="1:14">
+    <row r="259" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A259" t="s">
         <v>18</v>
       </c>
@@ -27134,7 +27158,7 @@
         <v>4994</v>
       </c>
     </row>
-    <row r="260" spans="1:14">
+    <row r="260" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A260" t="s">
         <v>14</v>
       </c>
@@ -27178,7 +27202,7 @@
         <v>4995</v>
       </c>
     </row>
-    <row r="261" spans="1:14">
+    <row r="261" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A261" t="s">
         <v>18</v>
       </c>
@@ -27222,7 +27246,7 @@
         <v>4996</v>
       </c>
     </row>
-    <row r="262" spans="1:14">
+    <row r="262" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A262" t="s">
         <v>14</v>
       </c>
@@ -27266,7 +27290,7 @@
         <v>4997</v>
       </c>
     </row>
-    <row r="263" spans="1:14">
+    <row r="263" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A263" t="s">
         <v>18</v>
       </c>
@@ -27310,7 +27334,7 @@
         <v>4998</v>
       </c>
     </row>
-    <row r="264" spans="1:14">
+    <row r="264" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A264" t="s">
         <v>14</v>
       </c>
@@ -27354,7 +27378,7 @@
         <v>4999</v>
       </c>
     </row>
-    <row r="265" spans="1:14">
+    <row r="265" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A265" t="s">
         <v>19</v>
       </c>
@@ -27398,7 +27422,7 @@
         <v>5000</v>
       </c>
     </row>
-    <row r="266" spans="1:14">
+    <row r="266" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A266" t="s">
         <v>14</v>
       </c>
@@ -27442,7 +27466,7 @@
         <v>5001</v>
       </c>
     </row>
-    <row r="267" spans="1:14">
+    <row r="267" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A267" t="s">
         <v>14</v>
       </c>
@@ -27486,7 +27510,7 @@
         <v>5002</v>
       </c>
     </row>
-    <row r="268" spans="1:14">
+    <row r="268" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A268" t="s">
         <v>14</v>
       </c>
@@ -27530,7 +27554,7 @@
         <v>5003</v>
       </c>
     </row>
-    <row r="269" spans="1:14">
+    <row r="269" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A269" t="s">
         <v>14</v>
       </c>
@@ -27574,7 +27598,7 @@
         <v>5004</v>
       </c>
     </row>
-    <row r="270" spans="1:14">
+    <row r="270" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A270" t="s">
         <v>16</v>
       </c>
@@ -27618,7 +27642,7 @@
         <v>5005</v>
       </c>
     </row>
-    <row r="271" spans="1:14">
+    <row r="271" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A271" t="s">
         <v>14</v>
       </c>
@@ -27662,7 +27686,7 @@
         <v>5006</v>
       </c>
     </row>
-    <row r="272" spans="1:14">
+    <row r="272" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A272" t="s">
         <v>14</v>
       </c>
@@ -27706,7 +27730,7 @@
         <v>5007</v>
       </c>
     </row>
-    <row r="273" spans="1:14">
+    <row r="273" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A273" t="s">
         <v>18</v>
       </c>
@@ -27750,7 +27774,7 @@
         <v>5008</v>
       </c>
     </row>
-    <row r="274" spans="1:14">
+    <row r="274" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A274" t="s">
         <v>16</v>
       </c>
@@ -27794,7 +27818,7 @@
         <v>5009</v>
       </c>
     </row>
-    <row r="275" spans="1:14">
+    <row r="275" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A275" t="s">
         <v>14</v>
       </c>
@@ -27838,7 +27862,7 @@
         <v>5010</v>
       </c>
     </row>
-    <row r="276" spans="1:14">
+    <row r="276" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A276" t="s">
         <v>18</v>
       </c>
@@ -27882,7 +27906,7 @@
         <v>5011</v>
       </c>
     </row>
-    <row r="277" spans="1:14">
+    <row r="277" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A277" t="s">
         <v>14</v>
       </c>
@@ -27926,7 +27950,7 @@
         <v>5012</v>
       </c>
     </row>
-    <row r="278" spans="1:14">
+    <row r="278" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A278" t="s">
         <v>14</v>
       </c>
@@ -27970,7 +27994,7 @@
         <v>5013</v>
       </c>
     </row>
-    <row r="279" spans="1:14">
+    <row r="279" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A279" t="s">
         <v>14</v>
       </c>
@@ -28014,7 +28038,7 @@
         <v>5014</v>
       </c>
     </row>
-    <row r="280" spans="1:14">
+    <row r="280" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A280" t="s">
         <v>18</v>
       </c>
@@ -28058,7 +28082,7 @@
         <v>5015</v>
       </c>
     </row>
-    <row r="281" spans="1:14">
+    <row r="281" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A281" t="s">
         <v>15</v>
       </c>
@@ -28102,7 +28126,7 @@
         <v>5016</v>
       </c>
     </row>
-    <row r="282" spans="1:14">
+    <row r="282" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A282" t="s">
         <v>16</v>
       </c>
@@ -28146,7 +28170,7 @@
         <v>5017</v>
       </c>
     </row>
-    <row r="283" spans="1:14">
+    <row r="283" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A283" t="s">
         <v>18</v>
       </c>
@@ -28190,7 +28214,7 @@
         <v>5018</v>
       </c>
     </row>
-    <row r="284" spans="1:14">
+    <row r="284" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A284" t="s">
         <v>14</v>
       </c>
@@ -28234,7 +28258,7 @@
         <v>5019</v>
       </c>
     </row>
-    <row r="285" spans="1:14">
+    <row r="285" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A285" t="s">
         <v>18</v>
       </c>
@@ -28278,7 +28302,7 @@
         <v>5020</v>
       </c>
     </row>
-    <row r="286" spans="1:14">
+    <row r="286" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A286" t="s">
         <v>14</v>
       </c>
@@ -28322,7 +28346,7 @@
         <v>5021</v>
       </c>
     </row>
-    <row r="287" spans="1:14">
+    <row r="287" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A287" t="s">
         <v>14</v>
       </c>
@@ -28366,7 +28390,7 @@
         <v>5022</v>
       </c>
     </row>
-    <row r="288" spans="1:14">
+    <row r="288" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A288" t="s">
         <v>14</v>
       </c>
@@ -28410,7 +28434,7 @@
         <v>5023</v>
       </c>
     </row>
-    <row r="289" spans="1:14">
+    <row r="289" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A289" t="s">
         <v>14</v>
       </c>
@@ -28454,7 +28478,7 @@
         <v>5024</v>
       </c>
     </row>
-    <row r="290" spans="1:14">
+    <row r="290" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A290" t="s">
         <v>14</v>
       </c>
@@ -28498,7 +28522,7 @@
         <v>5025</v>
       </c>
     </row>
-    <row r="291" spans="1:14">
+    <row r="291" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A291" t="s">
         <v>18</v>
       </c>
@@ -28542,7 +28566,7 @@
         <v>5026</v>
       </c>
     </row>
-    <row r="292" spans="1:14">
+    <row r="292" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A292" t="s">
         <v>14</v>
       </c>
@@ -28586,7 +28610,7 @@
         <v>5027</v>
       </c>
     </row>
-    <row r="293" spans="1:14">
+    <row r="293" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A293" t="s">
         <v>14</v>
       </c>
@@ -28630,7 +28654,7 @@
         <v>5028</v>
       </c>
     </row>
-    <row r="294" spans="1:14">
+    <row r="294" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A294" t="s">
         <v>18</v>
       </c>
@@ -28674,7 +28698,7 @@
         <v>5029</v>
       </c>
     </row>
-    <row r="295" spans="1:14">
+    <row r="295" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A295" t="s">
         <v>14</v>
       </c>
@@ -28718,7 +28742,7 @@
         <v>5030</v>
       </c>
     </row>
-    <row r="296" spans="1:14">
+    <row r="296" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A296" t="s">
         <v>14</v>
       </c>
@@ -28762,7 +28786,7 @@
         <v>5031</v>
       </c>
     </row>
-    <row r="297" spans="1:14">
+    <row r="297" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A297" t="s">
         <v>20</v>
       </c>
@@ -28806,7 +28830,7 @@
         <v>5032</v>
       </c>
     </row>
-    <row r="298" spans="1:14">
+    <row r="298" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A298" t="s">
         <v>14</v>
       </c>
@@ -28850,7 +28874,7 @@
         <v>5033</v>
       </c>
     </row>
-    <row r="299" spans="1:14">
+    <row r="299" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A299" t="s">
         <v>16</v>
       </c>
@@ -28894,7 +28918,7 @@
         <v>5034</v>
       </c>
     </row>
-    <row r="300" spans="1:14">
+    <row r="300" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A300" t="s">
         <v>14</v>
       </c>
@@ -28938,7 +28962,7 @@
         <v>5035</v>
       </c>
     </row>
-    <row r="301" spans="1:14">
+    <row r="301" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A301" t="s">
         <v>18</v>
       </c>
@@ -28982,7 +29006,7 @@
         <v>5036</v>
       </c>
     </row>
-    <row r="302" spans="1:14">
+    <row r="302" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A302" t="s">
         <v>19</v>
       </c>
@@ -29026,7 +29050,7 @@
         <v>5037</v>
       </c>
     </row>
-    <row r="303" spans="1:14">
+    <row r="303" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A303" t="s">
         <v>14</v>
       </c>
@@ -29070,7 +29094,7 @@
         <v>5038</v>
       </c>
     </row>
-    <row r="304" spans="1:14">
+    <row r="304" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A304" t="s">
         <v>14</v>
       </c>
@@ -29114,7 +29138,7 @@
         <v>5039</v>
       </c>
     </row>
-    <row r="305" spans="1:14">
+    <row r="305" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A305" t="s">
         <v>16</v>
       </c>
@@ -29158,7 +29182,7 @@
         <v>5040</v>
       </c>
     </row>
-    <row r="306" spans="1:14">
+    <row r="306" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A306" t="s">
         <v>14</v>
       </c>
@@ -29202,7 +29226,7 @@
         <v>5041</v>
       </c>
     </row>
-    <row r="307" spans="1:14">
+    <row r="307" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A307" t="s">
         <v>14</v>
       </c>
@@ -29246,7 +29270,7 @@
         <v>5042</v>
       </c>
     </row>
-    <row r="308" spans="1:14">
+    <row r="308" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A308" t="s">
         <v>14</v>
       </c>
@@ -29290,7 +29314,7 @@
         <v>5043</v>
       </c>
     </row>
-    <row r="309" spans="1:14">
+    <row r="309" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A309" t="s">
         <v>14</v>
       </c>
@@ -29334,7 +29358,7 @@
         <v>5044</v>
       </c>
     </row>
-    <row r="310" spans="1:14">
+    <row r="310" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A310" t="s">
         <v>18</v>
       </c>
@@ -29378,7 +29402,7 @@
         <v>5045</v>
       </c>
     </row>
-    <row r="311" spans="1:14">
+    <row r="311" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A311" t="s">
         <v>18</v>
       </c>
@@ -29422,7 +29446,7 @@
         <v>5046</v>
       </c>
     </row>
-    <row r="312" spans="1:14">
+    <row r="312" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A312" t="s">
         <v>18</v>
       </c>
@@ -29466,7 +29490,7 @@
         <v>5047</v>
       </c>
     </row>
-    <row r="313" spans="1:14">
+    <row r="313" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A313" t="s">
         <v>14</v>
       </c>
@@ -29510,7 +29534,7 @@
         <v>5048</v>
       </c>
     </row>
-    <row r="314" spans="1:14">
+    <row r="314" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A314" t="s">
         <v>14</v>
       </c>
@@ -29554,7 +29578,7 @@
         <v>5049</v>
       </c>
     </row>
-    <row r="315" spans="1:14">
+    <row r="315" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A315" t="s">
         <v>20</v>
       </c>
@@ -29598,7 +29622,7 @@
         <v>5050</v>
       </c>
     </row>
-    <row r="316" spans="1:14">
+    <row r="316" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A316" t="s">
         <v>14</v>
       </c>
@@ -29642,7 +29666,7 @@
         <v>5051</v>
       </c>
     </row>
-    <row r="317" spans="1:14">
+    <row r="317" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A317" t="s">
         <v>20</v>
       </c>
@@ -29686,7 +29710,7 @@
         <v>5052</v>
       </c>
     </row>
-    <row r="318" spans="1:14">
+    <row r="318" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A318" t="s">
         <v>14</v>
       </c>
@@ -29730,7 +29754,7 @@
         <v>5053</v>
       </c>
     </row>
-    <row r="319" spans="1:14">
+    <row r="319" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A319" t="s">
         <v>16</v>
       </c>
@@ -29774,7 +29798,7 @@
         <v>5054</v>
       </c>
     </row>
-    <row r="320" spans="1:14">
+    <row r="320" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A320" t="s">
         <v>18</v>
       </c>
@@ -29818,7 +29842,7 @@
         <v>5055</v>
       </c>
     </row>
-    <row r="321" spans="1:14">
+    <row r="321" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A321" t="s">
         <v>14</v>
       </c>
@@ -29862,7 +29886,7 @@
         <v>5056</v>
       </c>
     </row>
-    <row r="322" spans="1:14">
+    <row r="322" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A322" t="s">
         <v>16</v>
       </c>
@@ -29906,7 +29930,7 @@
         <v>5057</v>
       </c>
     </row>
-    <row r="323" spans="1:14">
+    <row r="323" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A323" t="s">
         <v>14</v>
       </c>
@@ -29950,7 +29974,7 @@
         <v>5058</v>
       </c>
     </row>
-    <row r="324" spans="1:14">
+    <row r="324" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A324" t="s">
         <v>14</v>
       </c>
@@ -29994,7 +30018,7 @@
         <v>5059</v>
       </c>
     </row>
-    <row r="325" spans="1:14">
+    <row r="325" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A325" t="s">
         <v>14</v>
       </c>
@@ -30038,7 +30062,7 @@
         <v>5060</v>
       </c>
     </row>
-    <row r="326" spans="1:14">
+    <row r="326" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A326" t="s">
         <v>14</v>
       </c>
@@ -30082,7 +30106,7 @@
         <v>5061</v>
       </c>
     </row>
-    <row r="327" spans="1:14">
+    <row r="327" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A327" t="s">
         <v>14</v>
       </c>
@@ -30126,7 +30150,7 @@
         <v>5062</v>
       </c>
     </row>
-    <row r="328" spans="1:14">
+    <row r="328" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A328" t="s">
         <v>17</v>
       </c>
@@ -30170,7 +30194,7 @@
         <v>5063</v>
       </c>
     </row>
-    <row r="329" spans="1:14">
+    <row r="329" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A329" t="s">
         <v>18</v>
       </c>
@@ -30214,7 +30238,7 @@
         <v>5064</v>
       </c>
     </row>
-    <row r="330" spans="1:14">
+    <row r="330" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A330" t="s">
         <v>18</v>
       </c>
@@ -30258,7 +30282,7 @@
         <v>5065</v>
       </c>
     </row>
-    <row r="331" spans="1:14">
+    <row r="331" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A331" t="s">
         <v>14</v>
       </c>
@@ -30302,7 +30326,7 @@
         <v>5066</v>
       </c>
     </row>
-    <row r="332" spans="1:14">
+    <row r="332" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A332" t="s">
         <v>17</v>
       </c>
@@ -30346,7 +30370,7 @@
         <v>5067</v>
       </c>
     </row>
-    <row r="333" spans="1:14">
+    <row r="333" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A333" t="s">
         <v>17</v>
       </c>
@@ -30390,7 +30414,7 @@
         <v>5068</v>
       </c>
     </row>
-    <row r="334" spans="1:14">
+    <row r="334" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A334" t="s">
         <v>15</v>
       </c>
@@ -30434,7 +30458,7 @@
         <v>5069</v>
       </c>
     </row>
-    <row r="335" spans="1:14">
+    <row r="335" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A335" t="s">
         <v>14</v>
       </c>
@@ -30478,7 +30502,7 @@
         <v>5070</v>
       </c>
     </row>
-    <row r="336" spans="1:14">
+    <row r="336" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A336" t="s">
         <v>14</v>
       </c>
@@ -30522,7 +30546,7 @@
         <v>5071</v>
       </c>
     </row>
-    <row r="337" spans="1:14">
+    <row r="337" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A337" t="s">
         <v>14</v>
       </c>
@@ -30566,7 +30590,7 @@
         <v>5072</v>
       </c>
     </row>
-    <row r="338" spans="1:14">
+    <row r="338" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A338" t="s">
         <v>20</v>
       </c>
@@ -30610,7 +30634,7 @@
         <v>5073</v>
       </c>
     </row>
-    <row r="339" spans="1:14">
+    <row r="339" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A339" t="s">
         <v>14</v>
       </c>
@@ -30654,7 +30678,7 @@
         <v>5074</v>
       </c>
     </row>
-    <row r="340" spans="1:14">
+    <row r="340" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A340" t="s">
         <v>15</v>
       </c>
@@ -30698,7 +30722,7 @@
         <v>5075</v>
       </c>
     </row>
-    <row r="341" spans="1:14">
+    <row r="341" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A341" t="s">
         <v>14</v>
       </c>
@@ -30742,7 +30766,7 @@
         <v>5076</v>
       </c>
     </row>
-    <row r="342" spans="1:14">
+    <row r="342" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A342" t="s">
         <v>18</v>
       </c>
@@ -30786,7 +30810,7 @@
         <v>5077</v>
       </c>
     </row>
-    <row r="343" spans="1:14">
+    <row r="343" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A343" t="s">
         <v>18</v>
       </c>
@@ -30830,7 +30854,7 @@
         <v>5078</v>
       </c>
     </row>
-    <row r="344" spans="1:14">
+    <row r="344" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A344" t="s">
         <v>14</v>
       </c>
@@ -30874,7 +30898,7 @@
         <v>5079</v>
       </c>
     </row>
-    <row r="345" spans="1:14">
+    <row r="345" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A345" t="s">
         <v>14</v>
       </c>
@@ -30918,7 +30942,7 @@
         <v>5080</v>
       </c>
     </row>
-    <row r="346" spans="1:14">
+    <row r="346" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A346" t="s">
         <v>18</v>
       </c>
@@ -30962,7 +30986,7 @@
         <v>5081</v>
       </c>
     </row>
-    <row r="347" spans="1:14">
+    <row r="347" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A347" t="s">
         <v>14</v>
       </c>
@@ -31006,7 +31030,7 @@
         <v>5082</v>
       </c>
     </row>
-    <row r="348" spans="1:14">
+    <row r="348" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A348" t="s">
         <v>15</v>
       </c>
@@ -31050,7 +31074,7 @@
         <v>5083</v>
       </c>
     </row>
-    <row r="349" spans="1:14">
+    <row r="349" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A349" t="s">
         <v>14</v>
       </c>
@@ -31094,7 +31118,7 @@
         <v>5084</v>
       </c>
     </row>
-    <row r="350" spans="1:14">
+    <row r="350" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A350" t="s">
         <v>18</v>
       </c>
@@ -31138,7 +31162,7 @@
         <v>5085</v>
       </c>
     </row>
-    <row r="351" spans="1:14">
+    <row r="351" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A351" t="s">
         <v>14</v>
       </c>
@@ -31182,7 +31206,7 @@
         <v>5086</v>
       </c>
     </row>
-    <row r="352" spans="1:14">
+    <row r="352" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A352" t="s">
         <v>14</v>
       </c>
@@ -31226,7 +31250,7 @@
         <v>5087</v>
       </c>
     </row>
-    <row r="353" spans="1:14">
+    <row r="353" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A353" t="s">
         <v>19</v>
       </c>
@@ -31270,7 +31294,7 @@
         <v>5088</v>
       </c>
     </row>
-    <row r="354" spans="1:14">
+    <row r="354" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A354" t="s">
         <v>16</v>
       </c>
@@ -31314,7 +31338,7 @@
         <v>5089</v>
       </c>
     </row>
-    <row r="355" spans="1:14">
+    <row r="355" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A355" t="s">
         <v>14</v>
       </c>
@@ -31358,7 +31382,7 @@
         <v>5090</v>
       </c>
     </row>
-    <row r="356" spans="1:14">
+    <row r="356" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A356" t="s">
         <v>14</v>
       </c>
@@ -31402,7 +31426,7 @@
         <v>5091</v>
       </c>
     </row>
-    <row r="357" spans="1:14">
+    <row r="357" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A357" t="s">
         <v>18</v>
       </c>
@@ -31446,7 +31470,7 @@
         <v>5092</v>
       </c>
     </row>
-    <row r="358" spans="1:14">
+    <row r="358" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A358" t="s">
         <v>14</v>
       </c>
@@ -31490,7 +31514,7 @@
         <v>5093</v>
       </c>
     </row>
-    <row r="359" spans="1:14">
+    <row r="359" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A359" t="s">
         <v>14</v>
       </c>
@@ -31534,7 +31558,7 @@
         <v>5094</v>
       </c>
     </row>
-    <row r="360" spans="1:14">
+    <row r="360" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A360" t="s">
         <v>18</v>
       </c>
@@ -31578,7 +31602,7 @@
         <v>5095</v>
       </c>
     </row>
-    <row r="361" spans="1:14">
+    <row r="361" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A361" t="s">
         <v>15</v>
       </c>
@@ -31622,7 +31646,7 @@
         <v>5096</v>
       </c>
     </row>
-    <row r="362" spans="1:14">
+    <row r="362" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A362" t="s">
         <v>18</v>
       </c>
@@ -31666,7 +31690,7 @@
         <v>5097</v>
       </c>
     </row>
-    <row r="363" spans="1:14">
+    <row r="363" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A363" t="s">
         <v>19</v>
       </c>
@@ -31710,7 +31734,7 @@
         <v>5098</v>
       </c>
     </row>
-    <row r="364" spans="1:14">
+    <row r="364" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A364" t="s">
         <v>14</v>
       </c>
@@ -31754,7 +31778,7 @@
         <v>5099</v>
       </c>
     </row>
-    <row r="365" spans="1:14">
+    <row r="365" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A365" t="s">
         <v>18</v>
       </c>
@@ -31798,7 +31822,7 @@
         <v>5100</v>
       </c>
     </row>
-    <row r="366" spans="1:14">
+    <row r="366" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A366" t="s">
         <v>16</v>
       </c>
@@ -31842,7 +31866,7 @@
         <v>5101</v>
       </c>
     </row>
-    <row r="367" spans="1:14">
+    <row r="367" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A367" t="s">
         <v>14</v>
       </c>
@@ -31886,7 +31910,7 @@
         <v>5102</v>
       </c>
     </row>
-    <row r="368" spans="1:14">
+    <row r="368" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A368" t="s">
         <v>14</v>
       </c>
@@ -31930,7 +31954,7 @@
         <v>5103</v>
       </c>
     </row>
-    <row r="369" spans="1:14">
+    <row r="369" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A369" t="s">
         <v>14</v>
       </c>
@@ -31974,7 +31998,7 @@
         <v>5104</v>
       </c>
     </row>
-    <row r="370" spans="1:14">
+    <row r="370" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A370" t="s">
         <v>14</v>
       </c>
@@ -32018,7 +32042,7 @@
         <v>5105</v>
       </c>
     </row>
-    <row r="371" spans="1:14">
+    <row r="371" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A371" t="s">
         <v>14</v>
       </c>
@@ -32062,7 +32086,7 @@
         <v>5106</v>
       </c>
     </row>
-    <row r="372" spans="1:14">
+    <row r="372" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A372" t="s">
         <v>14</v>
       </c>
@@ -32106,7 +32130,7 @@
         <v>5107</v>
       </c>
     </row>
-    <row r="373" spans="1:14">
+    <row r="373" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A373" t="s">
         <v>14</v>
       </c>
@@ -32150,7 +32174,7 @@
         <v>5108</v>
       </c>
     </row>
-    <row r="374" spans="1:14">
+    <row r="374" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A374" t="s">
         <v>17</v>
       </c>
@@ -32194,7 +32218,7 @@
         <v>5109</v>
       </c>
     </row>
-    <row r="375" spans="1:14">
+    <row r="375" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A375" t="s">
         <v>14</v>
       </c>
@@ -32238,7 +32262,7 @@
         <v>5110</v>
       </c>
     </row>
-    <row r="376" spans="1:14">
+    <row r="376" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A376" t="s">
         <v>20</v>
       </c>
@@ -32282,7 +32306,7 @@
         <v>5111</v>
       </c>
     </row>
-    <row r="377" spans="1:14">
+    <row r="377" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A377" t="s">
         <v>18</v>
       </c>
@@ -32326,7 +32350,7 @@
         <v>5112</v>
       </c>
     </row>
-    <row r="378" spans="1:14">
+    <row r="378" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A378" t="s">
         <v>17</v>
       </c>
@@ -32370,7 +32394,7 @@
         <v>5113</v>
       </c>
     </row>
-    <row r="379" spans="1:14">
+    <row r="379" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A379" t="s">
         <v>14</v>
       </c>
@@ -32414,7 +32438,7 @@
         <v>5114</v>
       </c>
     </row>
-    <row r="380" spans="1:14">
+    <row r="380" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A380" t="s">
         <v>16</v>
       </c>
@@ -32458,7 +32482,7 @@
         <v>5115</v>
       </c>
     </row>
-    <row r="381" spans="1:14">
+    <row r="381" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A381" t="s">
         <v>17</v>
       </c>
@@ -32502,7 +32526,7 @@
         <v>5116</v>
       </c>
     </row>
-    <row r="382" spans="1:14">
+    <row r="382" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A382" t="s">
         <v>14</v>
       </c>
@@ -32546,7 +32570,7 @@
         <v>5117</v>
       </c>
     </row>
-    <row r="383" spans="1:14">
+    <row r="383" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A383" t="s">
         <v>14</v>
       </c>
@@ -32590,7 +32614,7 @@
         <v>5118</v>
       </c>
     </row>
-    <row r="384" spans="1:14">
+    <row r="384" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A384" t="s">
         <v>18</v>
       </c>
@@ -32634,7 +32658,7 @@
         <v>5119</v>
       </c>
     </row>
-    <row r="385" spans="1:14">
+    <row r="385" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A385" t="s">
         <v>18</v>
       </c>
@@ -32678,7 +32702,7 @@
         <v>5120</v>
       </c>
     </row>
-    <row r="386" spans="1:14">
+    <row r="386" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A386" t="s">
         <v>20</v>
       </c>
@@ -32722,7 +32746,7 @@
         <v>5121</v>
       </c>
     </row>
-    <row r="387" spans="1:14">
+    <row r="387" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A387" t="s">
         <v>14</v>
       </c>
@@ -32766,7 +32790,7 @@
         <v>5122</v>
       </c>
     </row>
-    <row r="388" spans="1:14">
+    <row r="388" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A388" t="s">
         <v>18</v>
       </c>
@@ -32810,7 +32834,7 @@
         <v>5123</v>
       </c>
     </row>
-    <row r="389" spans="1:14">
+    <row r="389" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A389" t="s">
         <v>18</v>
       </c>
@@ -32854,7 +32878,7 @@
         <v>5124</v>
       </c>
     </row>
-    <row r="390" spans="1:14">
+    <row r="390" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A390" t="s">
         <v>14</v>
       </c>
@@ -32898,7 +32922,7 @@
         <v>5125</v>
       </c>
     </row>
-    <row r="391" spans="1:14">
+    <row r="391" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A391" t="s">
         <v>19</v>
       </c>
@@ -32942,7 +32966,7 @@
         <v>5126</v>
       </c>
     </row>
-    <row r="392" spans="1:14">
+    <row r="392" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A392" t="s">
         <v>14</v>
       </c>
@@ -32986,7 +33010,7 @@
         <v>5127</v>
       </c>
     </row>
-    <row r="393" spans="1:14">
+    <row r="393" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A393" t="s">
         <v>18</v>
       </c>
@@ -33030,7 +33054,7 @@
         <v>5128</v>
       </c>
     </row>
-    <row r="394" spans="1:14">
+    <row r="394" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A394" t="s">
         <v>19</v>
       </c>

</xml_diff>

<commit_message>
Adds the manual version 2 of better filtered/fine-tuned questions
</commit_message>
<xml_diff>
--- a/CCD-Bench/CCD-Bench_Business_V1.xlsx
+++ b/CCD-Bench/CCD-Bench_Business_V1.xlsx
@@ -1,21 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30026"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
   <workbookPr defaultThemeVersion="124226"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Data Storage\POLIMI\Semester 2\Multidisciplinary Project\LLM Culture Map Project\Code\CCD-Bench\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{34DD5D93-3CD6-429A-B31B-57D202AB4EAF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="124519"/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -15415,8 +15409,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <fonts count="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -15453,21 +15447,13 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2007 - 2010">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -15505,7 +15491,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2007 - 2010">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -15539,7 +15525,6 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -15574,10 +15559,9 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2007 - 2010">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -15750,19 +15734,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:N394"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="9.109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="187.88671875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="147" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="155.5546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="214.5546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="242.109375" bestFit="1" customWidth="1"/>
-  </cols>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:14">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -15806,7 +15782,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:14">
       <c r="A2" t="s">
         <v>14</v>
       </c>
@@ -15850,7 +15826,7 @@
         <v>4737</v>
       </c>
     </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:14">
       <c r="A3" t="s">
         <v>14</v>
       </c>
@@ -15894,7 +15870,7 @@
         <v>4738</v>
       </c>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:14">
       <c r="A4" t="s">
         <v>15</v>
       </c>
@@ -15938,7 +15914,7 @@
         <v>4739</v>
       </c>
     </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:14">
       <c r="A5" t="s">
         <v>14</v>
       </c>
@@ -15982,7 +15958,7 @@
         <v>4740</v>
       </c>
     </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:14">
       <c r="A6" t="s">
         <v>16</v>
       </c>
@@ -16026,7 +16002,7 @@
         <v>4741</v>
       </c>
     </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:14">
       <c r="A7" t="s">
         <v>14</v>
       </c>
@@ -16070,7 +16046,7 @@
         <v>4742</v>
       </c>
     </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:14">
       <c r="A8" t="s">
         <v>17</v>
       </c>
@@ -16114,7 +16090,7 @@
         <v>4743</v>
       </c>
     </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:14">
       <c r="A9" t="s">
         <v>14</v>
       </c>
@@ -16158,7 +16134,7 @@
         <v>4744</v>
       </c>
     </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:14">
       <c r="A10" t="s">
         <v>18</v>
       </c>
@@ -16202,7 +16178,7 @@
         <v>4745</v>
       </c>
     </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:14">
       <c r="A11" t="s">
         <v>14</v>
       </c>
@@ -16246,7 +16222,7 @@
         <v>4746</v>
       </c>
     </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:14">
       <c r="A12" t="s">
         <v>14</v>
       </c>
@@ -16290,7 +16266,7 @@
         <v>4747</v>
       </c>
     </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:14">
       <c r="A13" t="s">
         <v>14</v>
       </c>
@@ -16334,7 +16310,7 @@
         <v>4748</v>
       </c>
     </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:14">
       <c r="A14" t="s">
         <v>18</v>
       </c>
@@ -16378,7 +16354,7 @@
         <v>4749</v>
       </c>
     </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:14">
       <c r="A15" t="s">
         <v>19</v>
       </c>
@@ -16422,7 +16398,7 @@
         <v>4750</v>
       </c>
     </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:14">
       <c r="A16" t="s">
         <v>14</v>
       </c>
@@ -16466,7 +16442,7 @@
         <v>4751</v>
       </c>
     </row>
-    <row r="17" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:14">
       <c r="A17" t="s">
         <v>14</v>
       </c>
@@ -16510,7 +16486,7 @@
         <v>4752</v>
       </c>
     </row>
-    <row r="18" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:14">
       <c r="A18" t="s">
         <v>18</v>
       </c>
@@ -16554,7 +16530,7 @@
         <v>4753</v>
       </c>
     </row>
-    <row r="19" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:14">
       <c r="A19" t="s">
         <v>18</v>
       </c>
@@ -16598,7 +16574,7 @@
         <v>4754</v>
       </c>
     </row>
-    <row r="20" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:14">
       <c r="A20" t="s">
         <v>16</v>
       </c>
@@ -16642,7 +16618,7 @@
         <v>4755</v>
       </c>
     </row>
-    <row r="21" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:14">
       <c r="A21" t="s">
         <v>14</v>
       </c>
@@ -16686,7 +16662,7 @@
         <v>4756</v>
       </c>
     </row>
-    <row r="22" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:14">
       <c r="A22" t="s">
         <v>14</v>
       </c>
@@ -16730,7 +16706,7 @@
         <v>4757</v>
       </c>
     </row>
-    <row r="23" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:14">
       <c r="A23" t="s">
         <v>18</v>
       </c>
@@ -16774,7 +16750,7 @@
         <v>4758</v>
       </c>
     </row>
-    <row r="24" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:14">
       <c r="A24" t="s">
         <v>18</v>
       </c>
@@ -16818,7 +16794,7 @@
         <v>4759</v>
       </c>
     </row>
-    <row r="25" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:14">
       <c r="A25" t="s">
         <v>14</v>
       </c>
@@ -16862,7 +16838,7 @@
         <v>4760</v>
       </c>
     </row>
-    <row r="26" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:14">
       <c r="A26" t="s">
         <v>14</v>
       </c>
@@ -16906,7 +16882,7 @@
         <v>4761</v>
       </c>
     </row>
-    <row r="27" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:14">
       <c r="A27" t="s">
         <v>15</v>
       </c>
@@ -16950,7 +16926,7 @@
         <v>4762</v>
       </c>
     </row>
-    <row r="28" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:14">
       <c r="A28" t="s">
         <v>14</v>
       </c>
@@ -16994,7 +16970,7 @@
         <v>4763</v>
       </c>
     </row>
-    <row r="29" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:14">
       <c r="A29" t="s">
         <v>16</v>
       </c>
@@ -17038,7 +17014,7 @@
         <v>4764</v>
       </c>
     </row>
-    <row r="30" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:14">
       <c r="A30" t="s">
         <v>14</v>
       </c>
@@ -17082,7 +17058,7 @@
         <v>4765</v>
       </c>
     </row>
-    <row r="31" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:14">
       <c r="A31" t="s">
         <v>15</v>
       </c>
@@ -17126,7 +17102,7 @@
         <v>4766</v>
       </c>
     </row>
-    <row r="32" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:14">
       <c r="A32" t="s">
         <v>14</v>
       </c>
@@ -17170,7 +17146,7 @@
         <v>4767</v>
       </c>
     </row>
-    <row r="33" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:14">
       <c r="A33" t="s">
         <v>20</v>
       </c>
@@ -17214,7 +17190,7 @@
         <v>4768</v>
       </c>
     </row>
-    <row r="34" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:14">
       <c r="A34" t="s">
         <v>14</v>
       </c>
@@ -17258,7 +17234,7 @@
         <v>4769</v>
       </c>
     </row>
-    <row r="35" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:14">
       <c r="A35" t="s">
         <v>14</v>
       </c>
@@ -17302,7 +17278,7 @@
         <v>4770</v>
       </c>
     </row>
-    <row r="36" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:14">
       <c r="A36" t="s">
         <v>14</v>
       </c>
@@ -17346,7 +17322,7 @@
         <v>4771</v>
       </c>
     </row>
-    <row r="37" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:14">
       <c r="A37" t="s">
         <v>14</v>
       </c>
@@ -17390,7 +17366,7 @@
         <v>4772</v>
       </c>
     </row>
-    <row r="38" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:14">
       <c r="A38" t="s">
         <v>14</v>
       </c>
@@ -17434,7 +17410,7 @@
         <v>4773</v>
       </c>
     </row>
-    <row r="39" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:14">
       <c r="A39" t="s">
         <v>14</v>
       </c>
@@ -17478,7 +17454,7 @@
         <v>4774</v>
       </c>
     </row>
-    <row r="40" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:14">
       <c r="A40" t="s">
         <v>14</v>
       </c>
@@ -17522,7 +17498,7 @@
         <v>4775</v>
       </c>
     </row>
-    <row r="41" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:14">
       <c r="A41" t="s">
         <v>18</v>
       </c>
@@ -17566,7 +17542,7 @@
         <v>4776</v>
       </c>
     </row>
-    <row r="42" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:14">
       <c r="A42" t="s">
         <v>20</v>
       </c>
@@ -17610,7 +17586,7 @@
         <v>4777</v>
       </c>
     </row>
-    <row r="43" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:14">
       <c r="A43" t="s">
         <v>18</v>
       </c>
@@ -17654,7 +17630,7 @@
         <v>4778</v>
       </c>
     </row>
-    <row r="44" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:14">
       <c r="A44" t="s">
         <v>14</v>
       </c>
@@ -17698,7 +17674,7 @@
         <v>4779</v>
       </c>
     </row>
-    <row r="45" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:14">
       <c r="A45" t="s">
         <v>14</v>
       </c>
@@ -17742,7 +17718,7 @@
         <v>4780</v>
       </c>
     </row>
-    <row r="46" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:14">
       <c r="A46" t="s">
         <v>17</v>
       </c>
@@ -17786,7 +17762,7 @@
         <v>4781</v>
       </c>
     </row>
-    <row r="47" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:14">
       <c r="A47" t="s">
         <v>14</v>
       </c>
@@ -17830,7 +17806,7 @@
         <v>4782</v>
       </c>
     </row>
-    <row r="48" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:14">
       <c r="A48" t="s">
         <v>14</v>
       </c>
@@ -17874,7 +17850,7 @@
         <v>4783</v>
       </c>
     </row>
-    <row r="49" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:14">
       <c r="A49" t="s">
         <v>14</v>
       </c>
@@ -17918,7 +17894,7 @@
         <v>4784</v>
       </c>
     </row>
-    <row r="50" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:14">
       <c r="A50" t="s">
         <v>18</v>
       </c>
@@ -17962,7 +17938,7 @@
         <v>4785</v>
       </c>
     </row>
-    <row r="51" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:14">
       <c r="A51" t="s">
         <v>18</v>
       </c>
@@ -18006,7 +17982,7 @@
         <v>4786</v>
       </c>
     </row>
-    <row r="52" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:14">
       <c r="A52" t="s">
         <v>14</v>
       </c>
@@ -18050,7 +18026,7 @@
         <v>4787</v>
       </c>
     </row>
-    <row r="53" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:14">
       <c r="A53" t="s">
         <v>14</v>
       </c>
@@ -18094,7 +18070,7 @@
         <v>4788</v>
       </c>
     </row>
-    <row r="54" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:14">
       <c r="A54" t="s">
         <v>16</v>
       </c>
@@ -18138,7 +18114,7 @@
         <v>4789</v>
       </c>
     </row>
-    <row r="55" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:14">
       <c r="A55" t="s">
         <v>18</v>
       </c>
@@ -18182,7 +18158,7 @@
         <v>4790</v>
       </c>
     </row>
-    <row r="56" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:14">
       <c r="A56" t="s">
         <v>14</v>
       </c>
@@ -18226,7 +18202,7 @@
         <v>4791</v>
       </c>
     </row>
-    <row r="57" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:14">
       <c r="A57" t="s">
         <v>14</v>
       </c>
@@ -18270,7 +18246,7 @@
         <v>4792</v>
       </c>
     </row>
-    <row r="58" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:14">
       <c r="A58" t="s">
         <v>14</v>
       </c>
@@ -18314,7 +18290,7 @@
         <v>4793</v>
       </c>
     </row>
-    <row r="59" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:14">
       <c r="A59" t="s">
         <v>14</v>
       </c>
@@ -18358,7 +18334,7 @@
         <v>4794</v>
       </c>
     </row>
-    <row r="60" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:14">
       <c r="A60" t="s">
         <v>14</v>
       </c>
@@ -18402,7 +18378,7 @@
         <v>4795</v>
       </c>
     </row>
-    <row r="61" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:14">
       <c r="A61" t="s">
         <v>14</v>
       </c>
@@ -18446,7 +18422,7 @@
         <v>4796</v>
       </c>
     </row>
-    <row r="62" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:14">
       <c r="A62" t="s">
         <v>14</v>
       </c>
@@ -18490,7 +18466,7 @@
         <v>4797</v>
       </c>
     </row>
-    <row r="63" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:14">
       <c r="A63" t="s">
         <v>20</v>
       </c>
@@ -18534,7 +18510,7 @@
         <v>4798</v>
       </c>
     </row>
-    <row r="64" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:14">
       <c r="A64" t="s">
         <v>14</v>
       </c>
@@ -18578,7 +18554,7 @@
         <v>4799</v>
       </c>
     </row>
-    <row r="65" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:14">
       <c r="A65" t="s">
         <v>14</v>
       </c>
@@ -18622,7 +18598,7 @@
         <v>4800</v>
       </c>
     </row>
-    <row r="66" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:14">
       <c r="A66" t="s">
         <v>14</v>
       </c>
@@ -18666,7 +18642,7 @@
         <v>4801</v>
       </c>
     </row>
-    <row r="67" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:14">
       <c r="A67" t="s">
         <v>14</v>
       </c>
@@ -18710,7 +18686,7 @@
         <v>4802</v>
       </c>
     </row>
-    <row r="68" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:14">
       <c r="A68" t="s">
         <v>14</v>
       </c>
@@ -18754,7 +18730,7 @@
         <v>4803</v>
       </c>
     </row>
-    <row r="69" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:14">
       <c r="A69" t="s">
         <v>20</v>
       </c>
@@ -18798,7 +18774,7 @@
         <v>4804</v>
       </c>
     </row>
-    <row r="70" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:14">
       <c r="A70" t="s">
         <v>14</v>
       </c>
@@ -18842,7 +18818,7 @@
         <v>4805</v>
       </c>
     </row>
-    <row r="71" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:14">
       <c r="A71" t="s">
         <v>18</v>
       </c>
@@ -18886,7 +18862,7 @@
         <v>4806</v>
       </c>
     </row>
-    <row r="72" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:14">
       <c r="A72" t="s">
         <v>18</v>
       </c>
@@ -18930,7 +18906,7 @@
         <v>4807</v>
       </c>
     </row>
-    <row r="73" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:14">
       <c r="A73" t="s">
         <v>20</v>
       </c>
@@ -18974,7 +18950,7 @@
         <v>4808</v>
       </c>
     </row>
-    <row r="74" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:14">
       <c r="A74" t="s">
         <v>14</v>
       </c>
@@ -19018,7 +18994,7 @@
         <v>4809</v>
       </c>
     </row>
-    <row r="75" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:14">
       <c r="A75" t="s">
         <v>18</v>
       </c>
@@ -19062,7 +19038,7 @@
         <v>4810</v>
       </c>
     </row>
-    <row r="76" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:14">
       <c r="A76" t="s">
         <v>14</v>
       </c>
@@ -19106,7 +19082,7 @@
         <v>4811</v>
       </c>
     </row>
-    <row r="77" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:14">
       <c r="A77" t="s">
         <v>18</v>
       </c>
@@ -19150,7 +19126,7 @@
         <v>4812</v>
       </c>
     </row>
-    <row r="78" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:14">
       <c r="A78" t="s">
         <v>14</v>
       </c>
@@ -19194,7 +19170,7 @@
         <v>4813</v>
       </c>
     </row>
-    <row r="79" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:14">
       <c r="A79" t="s">
         <v>16</v>
       </c>
@@ -19238,7 +19214,7 @@
         <v>4814</v>
       </c>
     </row>
-    <row r="80" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:14">
       <c r="A80" t="s">
         <v>14</v>
       </c>
@@ -19282,7 +19258,7 @@
         <v>4815</v>
       </c>
     </row>
-    <row r="81" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:14">
       <c r="A81" t="s">
         <v>14</v>
       </c>
@@ -19326,7 +19302,7 @@
         <v>4816</v>
       </c>
     </row>
-    <row r="82" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:14">
       <c r="A82" t="s">
         <v>18</v>
       </c>
@@ -19370,7 +19346,7 @@
         <v>4817</v>
       </c>
     </row>
-    <row r="83" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:14">
       <c r="A83" t="s">
         <v>16</v>
       </c>
@@ -19414,7 +19390,7 @@
         <v>4818</v>
       </c>
     </row>
-    <row r="84" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:14">
       <c r="A84" t="s">
         <v>14</v>
       </c>
@@ -19458,7 +19434,7 @@
         <v>4819</v>
       </c>
     </row>
-    <row r="85" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:14">
       <c r="A85" t="s">
         <v>14</v>
       </c>
@@ -19502,7 +19478,7 @@
         <v>4820</v>
       </c>
     </row>
-    <row r="86" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:14">
       <c r="A86" t="s">
         <v>14</v>
       </c>
@@ -19546,7 +19522,7 @@
         <v>4821</v>
       </c>
     </row>
-    <row r="87" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:14">
       <c r="A87" t="s">
         <v>14</v>
       </c>
@@ -19590,7 +19566,7 @@
         <v>4822</v>
       </c>
     </row>
-    <row r="88" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:14">
       <c r="A88" t="s">
         <v>14</v>
       </c>
@@ -19634,7 +19610,7 @@
         <v>4823</v>
       </c>
     </row>
-    <row r="89" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:14">
       <c r="A89" t="s">
         <v>18</v>
       </c>
@@ -19678,7 +19654,7 @@
         <v>4824</v>
       </c>
     </row>
-    <row r="90" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:14">
       <c r="A90" t="s">
         <v>14</v>
       </c>
@@ -19722,7 +19698,7 @@
         <v>4825</v>
       </c>
     </row>
-    <row r="91" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:14">
       <c r="A91" t="s">
         <v>14</v>
       </c>
@@ -19766,7 +19742,7 @@
         <v>4826</v>
       </c>
     </row>
-    <row r="92" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:14">
       <c r="A92" t="s">
         <v>14</v>
       </c>
@@ -19810,7 +19786,7 @@
         <v>4827</v>
       </c>
     </row>
-    <row r="93" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:14">
       <c r="A93" t="s">
         <v>18</v>
       </c>
@@ -19854,7 +19830,7 @@
         <v>4828</v>
       </c>
     </row>
-    <row r="94" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:14">
       <c r="A94" t="s">
         <v>14</v>
       </c>
@@ -19898,7 +19874,7 @@
         <v>4829</v>
       </c>
     </row>
-    <row r="95" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:14">
       <c r="A95" t="s">
         <v>17</v>
       </c>
@@ -19942,7 +19918,7 @@
         <v>4830</v>
       </c>
     </row>
-    <row r="96" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:14">
       <c r="A96" t="s">
         <v>18</v>
       </c>
@@ -19986,7 +19962,7 @@
         <v>4831</v>
       </c>
     </row>
-    <row r="97" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:14">
       <c r="A97" t="s">
         <v>14</v>
       </c>
@@ -20030,7 +20006,7 @@
         <v>4832</v>
       </c>
     </row>
-    <row r="98" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:14">
       <c r="A98" t="s">
         <v>18</v>
       </c>
@@ -20074,7 +20050,7 @@
         <v>4833</v>
       </c>
     </row>
-    <row r="99" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:14">
       <c r="A99" t="s">
         <v>20</v>
       </c>
@@ -20118,7 +20094,7 @@
         <v>4834</v>
       </c>
     </row>
-    <row r="100" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:14">
       <c r="A100" t="s">
         <v>14</v>
       </c>
@@ -20162,7 +20138,7 @@
         <v>4835</v>
       </c>
     </row>
-    <row r="101" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:14">
       <c r="A101" t="s">
         <v>14</v>
       </c>
@@ -20206,7 +20182,7 @@
         <v>4836</v>
       </c>
     </row>
-    <row r="102" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:14">
       <c r="A102" t="s">
         <v>18</v>
       </c>
@@ -20250,7 +20226,7 @@
         <v>4837</v>
       </c>
     </row>
-    <row r="103" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:14">
       <c r="A103" t="s">
         <v>14</v>
       </c>
@@ -20294,7 +20270,7 @@
         <v>4838</v>
       </c>
     </row>
-    <row r="104" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:14">
       <c r="A104" t="s">
         <v>14</v>
       </c>
@@ -20338,7 +20314,7 @@
         <v>4839</v>
       </c>
     </row>
-    <row r="105" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:14">
       <c r="A105" t="s">
         <v>18</v>
       </c>
@@ -20382,7 +20358,7 @@
         <v>4840</v>
       </c>
     </row>
-    <row r="106" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:14">
       <c r="A106" t="s">
         <v>18</v>
       </c>
@@ -20426,7 +20402,7 @@
         <v>4841</v>
       </c>
     </row>
-    <row r="107" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:14">
       <c r="A107" t="s">
         <v>20</v>
       </c>
@@ -20470,7 +20446,7 @@
         <v>4842</v>
       </c>
     </row>
-    <row r="108" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:14">
       <c r="A108" t="s">
         <v>17</v>
       </c>
@@ -20514,7 +20490,7 @@
         <v>4843</v>
       </c>
     </row>
-    <row r="109" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:14">
       <c r="A109" t="s">
         <v>14</v>
       </c>
@@ -20558,7 +20534,7 @@
         <v>4844</v>
       </c>
     </row>
-    <row r="110" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:14">
       <c r="A110" t="s">
         <v>14</v>
       </c>
@@ -20602,7 +20578,7 @@
         <v>4845</v>
       </c>
     </row>
-    <row r="111" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:14">
       <c r="A111" t="s">
         <v>18</v>
       </c>
@@ -20646,7 +20622,7 @@
         <v>4846</v>
       </c>
     </row>
-    <row r="112" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:14">
       <c r="A112" t="s">
         <v>14</v>
       </c>
@@ -20690,7 +20666,7 @@
         <v>4847</v>
       </c>
     </row>
-    <row r="113" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:14">
       <c r="A113" t="s">
         <v>14</v>
       </c>
@@ -20734,7 +20710,7 @@
         <v>4848</v>
       </c>
     </row>
-    <row r="114" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:14">
       <c r="A114" t="s">
         <v>14</v>
       </c>
@@ -20778,7 +20754,7 @@
         <v>4849</v>
       </c>
     </row>
-    <row r="115" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:14">
       <c r="A115" t="s">
         <v>14</v>
       </c>
@@ -20822,7 +20798,7 @@
         <v>4850</v>
       </c>
     </row>
-    <row r="116" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:14">
       <c r="A116" t="s">
         <v>14</v>
       </c>
@@ -20866,7 +20842,7 @@
         <v>4851</v>
       </c>
     </row>
-    <row r="117" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:14">
       <c r="A117" t="s">
         <v>14</v>
       </c>
@@ -20910,7 +20886,7 @@
         <v>4852</v>
       </c>
     </row>
-    <row r="118" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:14">
       <c r="A118" t="s">
         <v>18</v>
       </c>
@@ -20954,7 +20930,7 @@
         <v>4853</v>
       </c>
     </row>
-    <row r="119" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:14">
       <c r="A119" t="s">
         <v>14</v>
       </c>
@@ -20998,7 +20974,7 @@
         <v>4854</v>
       </c>
     </row>
-    <row r="120" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:14">
       <c r="A120" t="s">
         <v>18</v>
       </c>
@@ -21042,7 +21018,7 @@
         <v>4855</v>
       </c>
     </row>
-    <row r="121" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:14">
       <c r="A121" t="s">
         <v>14</v>
       </c>
@@ -21086,7 +21062,7 @@
         <v>4856</v>
       </c>
     </row>
-    <row r="122" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:14">
       <c r="A122" t="s">
         <v>18</v>
       </c>
@@ -21130,7 +21106,7 @@
         <v>4857</v>
       </c>
     </row>
-    <row r="123" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:14">
       <c r="A123" t="s">
         <v>20</v>
       </c>
@@ -21174,7 +21150,7 @@
         <v>4858</v>
       </c>
     </row>
-    <row r="124" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:14">
       <c r="A124" t="s">
         <v>18</v>
       </c>
@@ -21218,7 +21194,7 @@
         <v>4859</v>
       </c>
     </row>
-    <row r="125" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:14">
       <c r="A125" t="s">
         <v>14</v>
       </c>
@@ -21262,7 +21238,7 @@
         <v>4860</v>
       </c>
     </row>
-    <row r="126" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:14">
       <c r="A126" t="s">
         <v>14</v>
       </c>
@@ -21306,7 +21282,7 @@
         <v>4861</v>
       </c>
     </row>
-    <row r="127" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:14">
       <c r="A127" t="s">
         <v>18</v>
       </c>
@@ -21350,7 +21326,7 @@
         <v>4862</v>
       </c>
     </row>
-    <row r="128" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:14">
       <c r="A128" t="s">
         <v>14</v>
       </c>
@@ -21394,7 +21370,7 @@
         <v>4863</v>
       </c>
     </row>
-    <row r="129" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:14">
       <c r="A129" t="s">
         <v>14</v>
       </c>
@@ -21438,7 +21414,7 @@
         <v>4864</v>
       </c>
     </row>
-    <row r="130" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:14">
       <c r="A130" t="s">
         <v>14</v>
       </c>
@@ -21482,7 +21458,7 @@
         <v>4865</v>
       </c>
     </row>
-    <row r="131" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:14">
       <c r="A131" t="s">
         <v>14</v>
       </c>
@@ -21526,7 +21502,7 @@
         <v>4866</v>
       </c>
     </row>
-    <row r="132" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:14">
       <c r="A132" t="s">
         <v>14</v>
       </c>
@@ -21570,7 +21546,7 @@
         <v>4867</v>
       </c>
     </row>
-    <row r="133" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:14">
       <c r="A133" t="s">
         <v>14</v>
       </c>
@@ -21614,7 +21590,7 @@
         <v>4868</v>
       </c>
     </row>
-    <row r="134" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:14">
       <c r="A134" t="s">
         <v>18</v>
       </c>
@@ -21658,7 +21634,7 @@
         <v>4869</v>
       </c>
     </row>
-    <row r="135" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:14">
       <c r="A135" t="s">
         <v>18</v>
       </c>
@@ -21702,7 +21678,7 @@
         <v>4870</v>
       </c>
     </row>
-    <row r="136" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:14">
       <c r="A136" t="s">
         <v>14</v>
       </c>
@@ -21746,7 +21722,7 @@
         <v>4871</v>
       </c>
     </row>
-    <row r="137" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:14">
       <c r="A137" t="s">
         <v>14</v>
       </c>
@@ -21790,7 +21766,7 @@
         <v>4872</v>
       </c>
     </row>
-    <row r="138" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:14">
       <c r="A138" t="s">
         <v>14</v>
       </c>
@@ -21834,7 +21810,7 @@
         <v>4873</v>
       </c>
     </row>
-    <row r="139" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="139" spans="1:14">
       <c r="A139" t="s">
         <v>18</v>
       </c>
@@ -21878,7 +21854,7 @@
         <v>4874</v>
       </c>
     </row>
-    <row r="140" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="140" spans="1:14">
       <c r="A140" t="s">
         <v>14</v>
       </c>
@@ -21922,7 +21898,7 @@
         <v>4875</v>
       </c>
     </row>
-    <row r="141" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="141" spans="1:14">
       <c r="A141" t="s">
         <v>14</v>
       </c>
@@ -21966,7 +21942,7 @@
         <v>4876</v>
       </c>
     </row>
-    <row r="142" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="142" spans="1:14">
       <c r="A142" t="s">
         <v>14</v>
       </c>
@@ -22010,7 +21986,7 @@
         <v>4877</v>
       </c>
     </row>
-    <row r="143" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="143" spans="1:14">
       <c r="A143" t="s">
         <v>14</v>
       </c>
@@ -22054,7 +22030,7 @@
         <v>4878</v>
       </c>
     </row>
-    <row r="144" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="144" spans="1:14">
       <c r="A144" t="s">
         <v>17</v>
       </c>
@@ -22098,7 +22074,7 @@
         <v>4879</v>
       </c>
     </row>
-    <row r="145" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="145" spans="1:14">
       <c r="A145" t="s">
         <v>18</v>
       </c>
@@ -22142,7 +22118,7 @@
         <v>4880</v>
       </c>
     </row>
-    <row r="146" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="146" spans="1:14">
       <c r="A146" t="s">
         <v>14</v>
       </c>
@@ -22186,7 +22162,7 @@
         <v>4881</v>
       </c>
     </row>
-    <row r="147" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="147" spans="1:14">
       <c r="A147" t="s">
         <v>14</v>
       </c>
@@ -22230,7 +22206,7 @@
         <v>4882</v>
       </c>
     </row>
-    <row r="148" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="148" spans="1:14">
       <c r="A148" t="s">
         <v>15</v>
       </c>
@@ -22274,7 +22250,7 @@
         <v>4883</v>
       </c>
     </row>
-    <row r="149" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="149" spans="1:14">
       <c r="A149" t="s">
         <v>18</v>
       </c>
@@ -22318,7 +22294,7 @@
         <v>4884</v>
       </c>
     </row>
-    <row r="150" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="150" spans="1:14">
       <c r="A150" t="s">
         <v>14</v>
       </c>
@@ -22362,7 +22338,7 @@
         <v>4885</v>
       </c>
     </row>
-    <row r="151" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="151" spans="1:14">
       <c r="A151" t="s">
         <v>18</v>
       </c>
@@ -22406,7 +22382,7 @@
         <v>4886</v>
       </c>
     </row>
-    <row r="152" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="152" spans="1:14">
       <c r="A152" t="s">
         <v>14</v>
       </c>
@@ -22450,7 +22426,7 @@
         <v>4887</v>
       </c>
     </row>
-    <row r="153" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="153" spans="1:14">
       <c r="A153" t="s">
         <v>14</v>
       </c>
@@ -22494,7 +22470,7 @@
         <v>4888</v>
       </c>
     </row>
-    <row r="154" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="154" spans="1:14">
       <c r="A154" t="s">
         <v>18</v>
       </c>
@@ -22538,7 +22514,7 @@
         <v>4889</v>
       </c>
     </row>
-    <row r="155" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="155" spans="1:14">
       <c r="A155" t="s">
         <v>20</v>
       </c>
@@ -22582,7 +22558,7 @@
         <v>4890</v>
       </c>
     </row>
-    <row r="156" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="156" spans="1:14">
       <c r="A156" t="s">
         <v>18</v>
       </c>
@@ -22626,7 +22602,7 @@
         <v>4891</v>
       </c>
     </row>
-    <row r="157" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="157" spans="1:14">
       <c r="A157" t="s">
         <v>14</v>
       </c>
@@ -22670,7 +22646,7 @@
         <v>4892</v>
       </c>
     </row>
-    <row r="158" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="158" spans="1:14">
       <c r="A158" t="s">
         <v>20</v>
       </c>
@@ -22714,7 +22690,7 @@
         <v>4893</v>
       </c>
     </row>
-    <row r="159" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="159" spans="1:14">
       <c r="A159" t="s">
         <v>20</v>
       </c>
@@ -22758,7 +22734,7 @@
         <v>4894</v>
       </c>
     </row>
-    <row r="160" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="160" spans="1:14">
       <c r="A160" t="s">
         <v>14</v>
       </c>
@@ -22802,7 +22778,7 @@
         <v>4895</v>
       </c>
     </row>
-    <row r="161" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="161" spans="1:14">
       <c r="A161" t="s">
         <v>14</v>
       </c>
@@ -22846,7 +22822,7 @@
         <v>4896</v>
       </c>
     </row>
-    <row r="162" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="162" spans="1:14">
       <c r="A162" t="s">
         <v>14</v>
       </c>
@@ -22890,7 +22866,7 @@
         <v>4897</v>
       </c>
     </row>
-    <row r="163" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="163" spans="1:14">
       <c r="A163" t="s">
         <v>18</v>
       </c>
@@ -22934,7 +22910,7 @@
         <v>4898</v>
       </c>
     </row>
-    <row r="164" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="164" spans="1:14">
       <c r="A164" t="s">
         <v>18</v>
       </c>
@@ -22978,7 +22954,7 @@
         <v>4899</v>
       </c>
     </row>
-    <row r="165" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="165" spans="1:14">
       <c r="A165" t="s">
         <v>19</v>
       </c>
@@ -23022,7 +22998,7 @@
         <v>4900</v>
       </c>
     </row>
-    <row r="166" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="166" spans="1:14">
       <c r="A166" t="s">
         <v>14</v>
       </c>
@@ -23066,7 +23042,7 @@
         <v>4901</v>
       </c>
     </row>
-    <row r="167" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="167" spans="1:14">
       <c r="A167" t="s">
         <v>16</v>
       </c>
@@ -23110,7 +23086,7 @@
         <v>4902</v>
       </c>
     </row>
-    <row r="168" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="168" spans="1:14">
       <c r="A168" t="s">
         <v>14</v>
       </c>
@@ -23154,7 +23130,7 @@
         <v>4903</v>
       </c>
     </row>
-    <row r="169" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="169" spans="1:14">
       <c r="A169" t="s">
         <v>14</v>
       </c>
@@ -23198,7 +23174,7 @@
         <v>4904</v>
       </c>
     </row>
-    <row r="170" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="170" spans="1:14">
       <c r="A170" t="s">
         <v>14</v>
       </c>
@@ -23242,7 +23218,7 @@
         <v>4905</v>
       </c>
     </row>
-    <row r="171" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="171" spans="1:14">
       <c r="A171" t="s">
         <v>18</v>
       </c>
@@ -23286,7 +23262,7 @@
         <v>4906</v>
       </c>
     </row>
-    <row r="172" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="172" spans="1:14">
       <c r="A172" t="s">
         <v>18</v>
       </c>
@@ -23330,7 +23306,7 @@
         <v>4907</v>
       </c>
     </row>
-    <row r="173" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="173" spans="1:14">
       <c r="A173" t="s">
         <v>14</v>
       </c>
@@ -23374,7 +23350,7 @@
         <v>4908</v>
       </c>
     </row>
-    <row r="174" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="174" spans="1:14">
       <c r="A174" t="s">
         <v>14</v>
       </c>
@@ -23418,7 +23394,7 @@
         <v>4909</v>
       </c>
     </row>
-    <row r="175" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="175" spans="1:14">
       <c r="A175" t="s">
         <v>14</v>
       </c>
@@ -23462,7 +23438,7 @@
         <v>4910</v>
       </c>
     </row>
-    <row r="176" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="176" spans="1:14">
       <c r="A176" t="s">
         <v>14</v>
       </c>
@@ -23506,7 +23482,7 @@
         <v>4911</v>
       </c>
     </row>
-    <row r="177" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="177" spans="1:14">
       <c r="A177" t="s">
         <v>14</v>
       </c>
@@ -23550,7 +23526,7 @@
         <v>4912</v>
       </c>
     </row>
-    <row r="178" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="178" spans="1:14">
       <c r="A178" t="s">
         <v>14</v>
       </c>
@@ -23594,7 +23570,7 @@
         <v>4913</v>
       </c>
     </row>
-    <row r="179" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="179" spans="1:14">
       <c r="A179" t="s">
         <v>14</v>
       </c>
@@ -23638,7 +23614,7 @@
         <v>4914</v>
       </c>
     </row>
-    <row r="180" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="180" spans="1:14">
       <c r="A180" t="s">
         <v>14</v>
       </c>
@@ -23682,7 +23658,7 @@
         <v>4915</v>
       </c>
     </row>
-    <row r="181" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="181" spans="1:14">
       <c r="A181" t="s">
         <v>19</v>
       </c>
@@ -23726,7 +23702,7 @@
         <v>4916</v>
       </c>
     </row>
-    <row r="182" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="182" spans="1:14">
       <c r="A182" t="s">
         <v>14</v>
       </c>
@@ -23770,7 +23746,7 @@
         <v>4917</v>
       </c>
     </row>
-    <row r="183" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="183" spans="1:14">
       <c r="A183" t="s">
         <v>18</v>
       </c>
@@ -23814,7 +23790,7 @@
         <v>4918</v>
       </c>
     </row>
-    <row r="184" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="184" spans="1:14">
       <c r="A184" t="s">
         <v>14</v>
       </c>
@@ -23858,7 +23834,7 @@
         <v>4919</v>
       </c>
     </row>
-    <row r="185" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="185" spans="1:14">
       <c r="A185" t="s">
         <v>14</v>
       </c>
@@ -23902,7 +23878,7 @@
         <v>4920</v>
       </c>
     </row>
-    <row r="186" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="186" spans="1:14">
       <c r="A186" t="s">
         <v>15</v>
       </c>
@@ -23946,7 +23922,7 @@
         <v>4921</v>
       </c>
     </row>
-    <row r="187" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="187" spans="1:14">
       <c r="A187" t="s">
         <v>16</v>
       </c>
@@ -23990,7 +23966,7 @@
         <v>4922</v>
       </c>
     </row>
-    <row r="188" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="188" spans="1:14">
       <c r="A188" t="s">
         <v>18</v>
       </c>
@@ -24034,7 +24010,7 @@
         <v>4923</v>
       </c>
     </row>
-    <row r="189" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="189" spans="1:14">
       <c r="A189" t="s">
         <v>19</v>
       </c>
@@ -24078,7 +24054,7 @@
         <v>4924</v>
       </c>
     </row>
-    <row r="190" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="190" spans="1:14">
       <c r="A190" t="s">
         <v>14</v>
       </c>
@@ -24122,7 +24098,7 @@
         <v>4925</v>
       </c>
     </row>
-    <row r="191" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="191" spans="1:14">
       <c r="A191" t="s">
         <v>14</v>
       </c>
@@ -24166,7 +24142,7 @@
         <v>4926</v>
       </c>
     </row>
-    <row r="192" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="192" spans="1:14">
       <c r="A192" t="s">
         <v>18</v>
       </c>
@@ -24210,7 +24186,7 @@
         <v>4927</v>
       </c>
     </row>
-    <row r="193" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="193" spans="1:14">
       <c r="A193" t="s">
         <v>14</v>
       </c>
@@ -24254,7 +24230,7 @@
         <v>4928</v>
       </c>
     </row>
-    <row r="194" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="194" spans="1:14">
       <c r="A194" t="s">
         <v>20</v>
       </c>
@@ -24298,7 +24274,7 @@
         <v>4929</v>
       </c>
     </row>
-    <row r="195" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="195" spans="1:14">
       <c r="A195" t="s">
         <v>14</v>
       </c>
@@ -24342,7 +24318,7 @@
         <v>4930</v>
       </c>
     </row>
-    <row r="196" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="196" spans="1:14">
       <c r="A196" t="s">
         <v>16</v>
       </c>
@@ -24386,7 +24362,7 @@
         <v>4931</v>
       </c>
     </row>
-    <row r="197" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="197" spans="1:14">
       <c r="A197" t="s">
         <v>14</v>
       </c>
@@ -24430,7 +24406,7 @@
         <v>4932</v>
       </c>
     </row>
-    <row r="198" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="198" spans="1:14">
       <c r="A198" t="s">
         <v>15</v>
       </c>
@@ -24474,7 +24450,7 @@
         <v>4933</v>
       </c>
     </row>
-    <row r="199" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="199" spans="1:14">
       <c r="A199" t="s">
         <v>14</v>
       </c>
@@ -24518,7 +24494,7 @@
         <v>4934</v>
       </c>
     </row>
-    <row r="200" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="200" spans="1:14">
       <c r="A200" t="s">
         <v>14</v>
       </c>
@@ -24562,7 +24538,7 @@
         <v>4935</v>
       </c>
     </row>
-    <row r="201" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="201" spans="1:14">
       <c r="A201" t="s">
         <v>14</v>
       </c>
@@ -24606,7 +24582,7 @@
         <v>4936</v>
       </c>
     </row>
-    <row r="202" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="202" spans="1:14">
       <c r="A202" t="s">
         <v>17</v>
       </c>
@@ -24650,7 +24626,7 @@
         <v>4937</v>
       </c>
     </row>
-    <row r="203" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="203" spans="1:14">
       <c r="A203" t="s">
         <v>14</v>
       </c>
@@ -24694,7 +24670,7 @@
         <v>4938</v>
       </c>
     </row>
-    <row r="204" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="204" spans="1:14">
       <c r="A204" t="s">
         <v>14</v>
       </c>
@@ -24738,7 +24714,7 @@
         <v>4939</v>
       </c>
     </row>
-    <row r="205" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="205" spans="1:14">
       <c r="A205" t="s">
         <v>18</v>
       </c>
@@ -24782,7 +24758,7 @@
         <v>4940</v>
       </c>
     </row>
-    <row r="206" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="206" spans="1:14">
       <c r="A206" t="s">
         <v>14</v>
       </c>
@@ -24826,7 +24802,7 @@
         <v>4941</v>
       </c>
     </row>
-    <row r="207" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="207" spans="1:14">
       <c r="A207" t="s">
         <v>14</v>
       </c>
@@ -24870,7 +24846,7 @@
         <v>4942</v>
       </c>
     </row>
-    <row r="208" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="208" spans="1:14">
       <c r="A208" t="s">
         <v>14</v>
       </c>
@@ -24914,7 +24890,7 @@
         <v>4943</v>
       </c>
     </row>
-    <row r="209" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="209" spans="1:14">
       <c r="A209" t="s">
         <v>14</v>
       </c>
@@ -24958,7 +24934,7 @@
         <v>4944</v>
       </c>
     </row>
-    <row r="210" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="210" spans="1:14">
       <c r="A210" t="s">
         <v>14</v>
       </c>
@@ -25002,7 +24978,7 @@
         <v>4945</v>
       </c>
     </row>
-    <row r="211" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="211" spans="1:14">
       <c r="A211" t="s">
         <v>14</v>
       </c>
@@ -25046,7 +25022,7 @@
         <v>4946</v>
       </c>
     </row>
-    <row r="212" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="212" spans="1:14">
       <c r="A212" t="s">
         <v>16</v>
       </c>
@@ -25090,7 +25066,7 @@
         <v>4947</v>
       </c>
     </row>
-    <row r="213" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="213" spans="1:14">
       <c r="A213" t="s">
         <v>20</v>
       </c>
@@ -25134,7 +25110,7 @@
         <v>4948</v>
       </c>
     </row>
-    <row r="214" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="214" spans="1:14">
       <c r="A214" t="s">
         <v>14</v>
       </c>
@@ -25178,7 +25154,7 @@
         <v>4949</v>
       </c>
     </row>
-    <row r="215" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="215" spans="1:14">
       <c r="A215" t="s">
         <v>15</v>
       </c>
@@ -25222,7 +25198,7 @@
         <v>4950</v>
       </c>
     </row>
-    <row r="216" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="216" spans="1:14">
       <c r="A216" t="s">
         <v>20</v>
       </c>
@@ -25266,7 +25242,7 @@
         <v>4951</v>
       </c>
     </row>
-    <row r="217" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="217" spans="1:14">
       <c r="A217" t="s">
         <v>14</v>
       </c>
@@ -25310,7 +25286,7 @@
         <v>4952</v>
       </c>
     </row>
-    <row r="218" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="218" spans="1:14">
       <c r="A218" t="s">
         <v>14</v>
       </c>
@@ -25354,7 +25330,7 @@
         <v>4953</v>
       </c>
     </row>
-    <row r="219" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="219" spans="1:14">
       <c r="A219" t="s">
         <v>18</v>
       </c>
@@ -25398,7 +25374,7 @@
         <v>4954</v>
       </c>
     </row>
-    <row r="220" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="220" spans="1:14">
       <c r="A220" t="s">
         <v>14</v>
       </c>
@@ -25442,7 +25418,7 @@
         <v>4955</v>
       </c>
     </row>
-    <row r="221" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="221" spans="1:14">
       <c r="A221" t="s">
         <v>14</v>
       </c>
@@ -25486,7 +25462,7 @@
         <v>4956</v>
       </c>
     </row>
-    <row r="222" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="222" spans="1:14">
       <c r="A222" t="s">
         <v>14</v>
       </c>
@@ -25530,7 +25506,7 @@
         <v>4957</v>
       </c>
     </row>
-    <row r="223" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="223" spans="1:14">
       <c r="A223" t="s">
         <v>14</v>
       </c>
@@ -25574,7 +25550,7 @@
         <v>4958</v>
       </c>
     </row>
-    <row r="224" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="224" spans="1:14">
       <c r="A224" t="s">
         <v>18</v>
       </c>
@@ -25618,7 +25594,7 @@
         <v>4959</v>
       </c>
     </row>
-    <row r="225" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="225" spans="1:14">
       <c r="A225" t="s">
         <v>14</v>
       </c>
@@ -25662,7 +25638,7 @@
         <v>4960</v>
       </c>
     </row>
-    <row r="226" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="226" spans="1:14">
       <c r="A226" t="s">
         <v>18</v>
       </c>
@@ -25706,7 +25682,7 @@
         <v>4961</v>
       </c>
     </row>
-    <row r="227" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="227" spans="1:14">
       <c r="A227" t="s">
         <v>18</v>
       </c>
@@ -25750,7 +25726,7 @@
         <v>4962</v>
       </c>
     </row>
-    <row r="228" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="228" spans="1:14">
       <c r="A228" t="s">
         <v>14</v>
       </c>
@@ -25794,7 +25770,7 @@
         <v>4963</v>
       </c>
     </row>
-    <row r="229" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="229" spans="1:14">
       <c r="A229" t="s">
         <v>14</v>
       </c>
@@ -25838,7 +25814,7 @@
         <v>4964</v>
       </c>
     </row>
-    <row r="230" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="230" spans="1:14">
       <c r="A230" t="s">
         <v>16</v>
       </c>
@@ -25882,7 +25858,7 @@
         <v>4965</v>
       </c>
     </row>
-    <row r="231" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="231" spans="1:14">
       <c r="A231" t="s">
         <v>14</v>
       </c>
@@ -25926,7 +25902,7 @@
         <v>4966</v>
       </c>
     </row>
-    <row r="232" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="232" spans="1:14">
       <c r="A232" t="s">
         <v>14</v>
       </c>
@@ -25970,7 +25946,7 @@
         <v>4967</v>
       </c>
     </row>
-    <row r="233" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="233" spans="1:14">
       <c r="A233" t="s">
         <v>14</v>
       </c>
@@ -26014,7 +25990,7 @@
         <v>4968</v>
       </c>
     </row>
-    <row r="234" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="234" spans="1:14">
       <c r="A234" t="s">
         <v>14</v>
       </c>
@@ -26058,7 +26034,7 @@
         <v>4969</v>
       </c>
     </row>
-    <row r="235" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="235" spans="1:14">
       <c r="A235" t="s">
         <v>14</v>
       </c>
@@ -26102,7 +26078,7 @@
         <v>4970</v>
       </c>
     </row>
-    <row r="236" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="236" spans="1:14">
       <c r="A236" t="s">
         <v>20</v>
       </c>
@@ -26146,7 +26122,7 @@
         <v>4971</v>
       </c>
     </row>
-    <row r="237" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="237" spans="1:14">
       <c r="A237" t="s">
         <v>14</v>
       </c>
@@ -26190,7 +26166,7 @@
         <v>4972</v>
       </c>
     </row>
-    <row r="238" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="238" spans="1:14">
       <c r="A238" t="s">
         <v>14</v>
       </c>
@@ -26234,7 +26210,7 @@
         <v>4973</v>
       </c>
     </row>
-    <row r="239" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="239" spans="1:14">
       <c r="A239" t="s">
         <v>18</v>
       </c>
@@ -26278,7 +26254,7 @@
         <v>4974</v>
       </c>
     </row>
-    <row r="240" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="240" spans="1:14">
       <c r="A240" t="s">
         <v>14</v>
       </c>
@@ -26322,7 +26298,7 @@
         <v>4975</v>
       </c>
     </row>
-    <row r="241" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="241" spans="1:14">
       <c r="A241" t="s">
         <v>19</v>
       </c>
@@ -26366,7 +26342,7 @@
         <v>4976</v>
       </c>
     </row>
-    <row r="242" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="242" spans="1:14">
       <c r="A242" t="s">
         <v>14</v>
       </c>
@@ -26410,7 +26386,7 @@
         <v>4977</v>
       </c>
     </row>
-    <row r="243" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="243" spans="1:14">
       <c r="A243" t="s">
         <v>14</v>
       </c>
@@ -26454,7 +26430,7 @@
         <v>4978</v>
       </c>
     </row>
-    <row r="244" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="244" spans="1:14">
       <c r="A244" t="s">
         <v>14</v>
       </c>
@@ -26498,7 +26474,7 @@
         <v>4979</v>
       </c>
     </row>
-    <row r="245" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="245" spans="1:14">
       <c r="A245" t="s">
         <v>18</v>
       </c>
@@ -26542,7 +26518,7 @@
         <v>4980</v>
       </c>
     </row>
-    <row r="246" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="246" spans="1:14">
       <c r="A246" t="s">
         <v>14</v>
       </c>
@@ -26586,7 +26562,7 @@
         <v>4981</v>
       </c>
     </row>
-    <row r="247" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="247" spans="1:14">
       <c r="A247" t="s">
         <v>15</v>
       </c>
@@ -26630,7 +26606,7 @@
         <v>4982</v>
       </c>
     </row>
-    <row r="248" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="248" spans="1:14">
       <c r="A248" t="s">
         <v>18</v>
       </c>
@@ -26674,7 +26650,7 @@
         <v>4983</v>
       </c>
     </row>
-    <row r="249" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="249" spans="1:14">
       <c r="A249" t="s">
         <v>20</v>
       </c>
@@ -26718,7 +26694,7 @@
         <v>4984</v>
       </c>
     </row>
-    <row r="250" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="250" spans="1:14">
       <c r="A250" t="s">
         <v>18</v>
       </c>
@@ -26762,7 +26738,7 @@
         <v>4985</v>
       </c>
     </row>
-    <row r="251" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="251" spans="1:14">
       <c r="A251" t="s">
         <v>14</v>
       </c>
@@ -26806,7 +26782,7 @@
         <v>4986</v>
       </c>
     </row>
-    <row r="252" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="252" spans="1:14">
       <c r="A252" t="s">
         <v>14</v>
       </c>
@@ -26850,7 +26826,7 @@
         <v>4987</v>
       </c>
     </row>
-    <row r="253" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="253" spans="1:14">
       <c r="A253" t="s">
         <v>17</v>
       </c>
@@ -26894,7 +26870,7 @@
         <v>4988</v>
       </c>
     </row>
-    <row r="254" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="254" spans="1:14">
       <c r="A254" t="s">
         <v>20</v>
       </c>
@@ -26938,7 +26914,7 @@
         <v>4989</v>
       </c>
     </row>
-    <row r="255" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="255" spans="1:14">
       <c r="A255" t="s">
         <v>14</v>
       </c>
@@ -26982,7 +26958,7 @@
         <v>4990</v>
       </c>
     </row>
-    <row r="256" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="256" spans="1:14">
       <c r="A256" t="s">
         <v>14</v>
       </c>
@@ -27026,7 +27002,7 @@
         <v>4991</v>
       </c>
     </row>
-    <row r="257" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="257" spans="1:14">
       <c r="A257" t="s">
         <v>14</v>
       </c>
@@ -27070,7 +27046,7 @@
         <v>4992</v>
       </c>
     </row>
-    <row r="258" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="258" spans="1:14">
       <c r="A258" t="s">
         <v>14</v>
       </c>
@@ -27114,7 +27090,7 @@
         <v>4993</v>
       </c>
     </row>
-    <row r="259" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="259" spans="1:14">
       <c r="A259" t="s">
         <v>18</v>
       </c>
@@ -27158,7 +27134,7 @@
         <v>4994</v>
       </c>
     </row>
-    <row r="260" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="260" spans="1:14">
       <c r="A260" t="s">
         <v>14</v>
       </c>
@@ -27202,7 +27178,7 @@
         <v>4995</v>
       </c>
     </row>
-    <row r="261" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="261" spans="1:14">
       <c r="A261" t="s">
         <v>18</v>
       </c>
@@ -27246,7 +27222,7 @@
         <v>4996</v>
       </c>
     </row>
-    <row r="262" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="262" spans="1:14">
       <c r="A262" t="s">
         <v>14</v>
       </c>
@@ -27290,7 +27266,7 @@
         <v>4997</v>
       </c>
     </row>
-    <row r="263" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="263" spans="1:14">
       <c r="A263" t="s">
         <v>18</v>
       </c>
@@ -27334,7 +27310,7 @@
         <v>4998</v>
       </c>
     </row>
-    <row r="264" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="264" spans="1:14">
       <c r="A264" t="s">
         <v>14</v>
       </c>
@@ -27378,7 +27354,7 @@
         <v>4999</v>
       </c>
     </row>
-    <row r="265" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="265" spans="1:14">
       <c r="A265" t="s">
         <v>19</v>
       </c>
@@ -27422,7 +27398,7 @@
         <v>5000</v>
       </c>
     </row>
-    <row r="266" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="266" spans="1:14">
       <c r="A266" t="s">
         <v>14</v>
       </c>
@@ -27466,7 +27442,7 @@
         <v>5001</v>
       </c>
     </row>
-    <row r="267" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="267" spans="1:14">
       <c r="A267" t="s">
         <v>14</v>
       </c>
@@ -27510,7 +27486,7 @@
         <v>5002</v>
       </c>
     </row>
-    <row r="268" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="268" spans="1:14">
       <c r="A268" t="s">
         <v>14</v>
       </c>
@@ -27554,7 +27530,7 @@
         <v>5003</v>
       </c>
     </row>
-    <row r="269" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="269" spans="1:14">
       <c r="A269" t="s">
         <v>14</v>
       </c>
@@ -27598,7 +27574,7 @@
         <v>5004</v>
       </c>
     </row>
-    <row r="270" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="270" spans="1:14">
       <c r="A270" t="s">
         <v>16</v>
       </c>
@@ -27642,7 +27618,7 @@
         <v>5005</v>
       </c>
     </row>
-    <row r="271" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="271" spans="1:14">
       <c r="A271" t="s">
         <v>14</v>
       </c>
@@ -27686,7 +27662,7 @@
         <v>5006</v>
       </c>
     </row>
-    <row r="272" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="272" spans="1:14">
       <c r="A272" t="s">
         <v>14</v>
       </c>
@@ -27730,7 +27706,7 @@
         <v>5007</v>
       </c>
     </row>
-    <row r="273" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="273" spans="1:14">
       <c r="A273" t="s">
         <v>18</v>
       </c>
@@ -27774,7 +27750,7 @@
         <v>5008</v>
       </c>
     </row>
-    <row r="274" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="274" spans="1:14">
       <c r="A274" t="s">
         <v>16</v>
       </c>
@@ -27818,7 +27794,7 @@
         <v>5009</v>
       </c>
     </row>
-    <row r="275" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="275" spans="1:14">
       <c r="A275" t="s">
         <v>14</v>
       </c>
@@ -27862,7 +27838,7 @@
         <v>5010</v>
       </c>
     </row>
-    <row r="276" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="276" spans="1:14">
       <c r="A276" t="s">
         <v>18</v>
       </c>
@@ -27906,7 +27882,7 @@
         <v>5011</v>
       </c>
     </row>
-    <row r="277" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="277" spans="1:14">
       <c r="A277" t="s">
         <v>14</v>
       </c>
@@ -27950,7 +27926,7 @@
         <v>5012</v>
       </c>
     </row>
-    <row r="278" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="278" spans="1:14">
       <c r="A278" t="s">
         <v>14</v>
       </c>
@@ -27994,7 +27970,7 @@
         <v>5013</v>
       </c>
     </row>
-    <row r="279" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="279" spans="1:14">
       <c r="A279" t="s">
         <v>14</v>
       </c>
@@ -28038,7 +28014,7 @@
         <v>5014</v>
       </c>
     </row>
-    <row r="280" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="280" spans="1:14">
       <c r="A280" t="s">
         <v>18</v>
       </c>
@@ -28082,7 +28058,7 @@
         <v>5015</v>
       </c>
     </row>
-    <row r="281" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="281" spans="1:14">
       <c r="A281" t="s">
         <v>15</v>
       </c>
@@ -28126,7 +28102,7 @@
         <v>5016</v>
       </c>
     </row>
-    <row r="282" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="282" spans="1:14">
       <c r="A282" t="s">
         <v>16</v>
       </c>
@@ -28170,7 +28146,7 @@
         <v>5017</v>
       </c>
     </row>
-    <row r="283" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="283" spans="1:14">
       <c r="A283" t="s">
         <v>18</v>
       </c>
@@ -28214,7 +28190,7 @@
         <v>5018</v>
       </c>
     </row>
-    <row r="284" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="284" spans="1:14">
       <c r="A284" t="s">
         <v>14</v>
       </c>
@@ -28258,7 +28234,7 @@
         <v>5019</v>
       </c>
     </row>
-    <row r="285" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="285" spans="1:14">
       <c r="A285" t="s">
         <v>18</v>
       </c>
@@ -28302,7 +28278,7 @@
         <v>5020</v>
       </c>
     </row>
-    <row r="286" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="286" spans="1:14">
       <c r="A286" t="s">
         <v>14</v>
       </c>
@@ -28346,7 +28322,7 @@
         <v>5021</v>
       </c>
     </row>
-    <row r="287" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="287" spans="1:14">
       <c r="A287" t="s">
         <v>14</v>
       </c>
@@ -28390,7 +28366,7 @@
         <v>5022</v>
       </c>
     </row>
-    <row r="288" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="288" spans="1:14">
       <c r="A288" t="s">
         <v>14</v>
       </c>
@@ -28434,7 +28410,7 @@
         <v>5023</v>
       </c>
     </row>
-    <row r="289" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="289" spans="1:14">
       <c r="A289" t="s">
         <v>14</v>
       </c>
@@ -28478,7 +28454,7 @@
         <v>5024</v>
       </c>
     </row>
-    <row r="290" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="290" spans="1:14">
       <c r="A290" t="s">
         <v>14</v>
       </c>
@@ -28522,7 +28498,7 @@
         <v>5025</v>
       </c>
     </row>
-    <row r="291" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="291" spans="1:14">
       <c r="A291" t="s">
         <v>18</v>
       </c>
@@ -28566,7 +28542,7 @@
         <v>5026</v>
       </c>
     </row>
-    <row r="292" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="292" spans="1:14">
       <c r="A292" t="s">
         <v>14</v>
       </c>
@@ -28610,7 +28586,7 @@
         <v>5027</v>
       </c>
     </row>
-    <row r="293" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="293" spans="1:14">
       <c r="A293" t="s">
         <v>14</v>
       </c>
@@ -28654,7 +28630,7 @@
         <v>5028</v>
       </c>
     </row>
-    <row r="294" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="294" spans="1:14">
       <c r="A294" t="s">
         <v>18</v>
       </c>
@@ -28698,7 +28674,7 @@
         <v>5029</v>
       </c>
     </row>
-    <row r="295" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="295" spans="1:14">
       <c r="A295" t="s">
         <v>14</v>
       </c>
@@ -28742,7 +28718,7 @@
         <v>5030</v>
       </c>
     </row>
-    <row r="296" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="296" spans="1:14">
       <c r="A296" t="s">
         <v>14</v>
       </c>
@@ -28786,7 +28762,7 @@
         <v>5031</v>
       </c>
     </row>
-    <row r="297" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="297" spans="1:14">
       <c r="A297" t="s">
         <v>20</v>
       </c>
@@ -28830,7 +28806,7 @@
         <v>5032</v>
       </c>
     </row>
-    <row r="298" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="298" spans="1:14">
       <c r="A298" t="s">
         <v>14</v>
       </c>
@@ -28874,7 +28850,7 @@
         <v>5033</v>
       </c>
     </row>
-    <row r="299" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="299" spans="1:14">
       <c r="A299" t="s">
         <v>16</v>
       </c>
@@ -28918,7 +28894,7 @@
         <v>5034</v>
       </c>
     </row>
-    <row r="300" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="300" spans="1:14">
       <c r="A300" t="s">
         <v>14</v>
       </c>
@@ -28962,7 +28938,7 @@
         <v>5035</v>
       </c>
     </row>
-    <row r="301" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="301" spans="1:14">
       <c r="A301" t="s">
         <v>18</v>
       </c>
@@ -29006,7 +28982,7 @@
         <v>5036</v>
       </c>
     </row>
-    <row r="302" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="302" spans="1:14">
       <c r="A302" t="s">
         <v>19</v>
       </c>
@@ -29050,7 +29026,7 @@
         <v>5037</v>
       </c>
     </row>
-    <row r="303" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="303" spans="1:14">
       <c r="A303" t="s">
         <v>14</v>
       </c>
@@ -29094,7 +29070,7 @@
         <v>5038</v>
       </c>
     </row>
-    <row r="304" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="304" spans="1:14">
       <c r="A304" t="s">
         <v>14</v>
       </c>
@@ -29138,7 +29114,7 @@
         <v>5039</v>
       </c>
     </row>
-    <row r="305" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="305" spans="1:14">
       <c r="A305" t="s">
         <v>16</v>
       </c>
@@ -29182,7 +29158,7 @@
         <v>5040</v>
       </c>
     </row>
-    <row r="306" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="306" spans="1:14">
       <c r="A306" t="s">
         <v>14</v>
       </c>
@@ -29226,7 +29202,7 @@
         <v>5041</v>
       </c>
     </row>
-    <row r="307" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="307" spans="1:14">
       <c r="A307" t="s">
         <v>14</v>
       </c>
@@ -29270,7 +29246,7 @@
         <v>5042</v>
       </c>
     </row>
-    <row r="308" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="308" spans="1:14">
       <c r="A308" t="s">
         <v>14</v>
       </c>
@@ -29314,7 +29290,7 @@
         <v>5043</v>
       </c>
     </row>
-    <row r="309" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="309" spans="1:14">
       <c r="A309" t="s">
         <v>14</v>
       </c>
@@ -29358,7 +29334,7 @@
         <v>5044</v>
       </c>
     </row>
-    <row r="310" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="310" spans="1:14">
       <c r="A310" t="s">
         <v>18</v>
       </c>
@@ -29402,7 +29378,7 @@
         <v>5045</v>
       </c>
     </row>
-    <row r="311" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="311" spans="1:14">
       <c r="A311" t="s">
         <v>18</v>
       </c>
@@ -29446,7 +29422,7 @@
         <v>5046</v>
       </c>
     </row>
-    <row r="312" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="312" spans="1:14">
       <c r="A312" t="s">
         <v>18</v>
       </c>
@@ -29490,7 +29466,7 @@
         <v>5047</v>
       </c>
     </row>
-    <row r="313" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="313" spans="1:14">
       <c r="A313" t="s">
         <v>14</v>
       </c>
@@ -29534,7 +29510,7 @@
         <v>5048</v>
       </c>
     </row>
-    <row r="314" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="314" spans="1:14">
       <c r="A314" t="s">
         <v>14</v>
       </c>
@@ -29578,7 +29554,7 @@
         <v>5049</v>
       </c>
     </row>
-    <row r="315" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="315" spans="1:14">
       <c r="A315" t="s">
         <v>20</v>
       </c>
@@ -29622,7 +29598,7 @@
         <v>5050</v>
       </c>
     </row>
-    <row r="316" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="316" spans="1:14">
       <c r="A316" t="s">
         <v>14</v>
       </c>
@@ -29666,7 +29642,7 @@
         <v>5051</v>
       </c>
     </row>
-    <row r="317" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="317" spans="1:14">
       <c r="A317" t="s">
         <v>20</v>
       </c>
@@ -29710,7 +29686,7 @@
         <v>5052</v>
       </c>
     </row>
-    <row r="318" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="318" spans="1:14">
       <c r="A318" t="s">
         <v>14</v>
       </c>
@@ -29754,7 +29730,7 @@
         <v>5053</v>
       </c>
     </row>
-    <row r="319" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="319" spans="1:14">
       <c r="A319" t="s">
         <v>16</v>
       </c>
@@ -29798,7 +29774,7 @@
         <v>5054</v>
       </c>
     </row>
-    <row r="320" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="320" spans="1:14">
       <c r="A320" t="s">
         <v>18</v>
       </c>
@@ -29842,7 +29818,7 @@
         <v>5055</v>
       </c>
     </row>
-    <row r="321" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="321" spans="1:14">
       <c r="A321" t="s">
         <v>14</v>
       </c>
@@ -29886,7 +29862,7 @@
         <v>5056</v>
       </c>
     </row>
-    <row r="322" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="322" spans="1:14">
       <c r="A322" t="s">
         <v>16</v>
       </c>
@@ -29930,7 +29906,7 @@
         <v>5057</v>
       </c>
     </row>
-    <row r="323" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="323" spans="1:14">
       <c r="A323" t="s">
         <v>14</v>
       </c>
@@ -29974,7 +29950,7 @@
         <v>5058</v>
       </c>
     </row>
-    <row r="324" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="324" spans="1:14">
       <c r="A324" t="s">
         <v>14</v>
       </c>
@@ -30018,7 +29994,7 @@
         <v>5059</v>
       </c>
     </row>
-    <row r="325" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="325" spans="1:14">
       <c r="A325" t="s">
         <v>14</v>
       </c>
@@ -30062,7 +30038,7 @@
         <v>5060</v>
       </c>
     </row>
-    <row r="326" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="326" spans="1:14">
       <c r="A326" t="s">
         <v>14</v>
       </c>
@@ -30106,7 +30082,7 @@
         <v>5061</v>
       </c>
     </row>
-    <row r="327" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="327" spans="1:14">
       <c r="A327" t="s">
         <v>14</v>
       </c>
@@ -30150,7 +30126,7 @@
         <v>5062</v>
       </c>
     </row>
-    <row r="328" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="328" spans="1:14">
       <c r="A328" t="s">
         <v>17</v>
       </c>
@@ -30194,7 +30170,7 @@
         <v>5063</v>
       </c>
     </row>
-    <row r="329" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="329" spans="1:14">
       <c r="A329" t="s">
         <v>18</v>
       </c>
@@ -30238,7 +30214,7 @@
         <v>5064</v>
       </c>
     </row>
-    <row r="330" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="330" spans="1:14">
       <c r="A330" t="s">
         <v>18</v>
       </c>
@@ -30282,7 +30258,7 @@
         <v>5065</v>
       </c>
     </row>
-    <row r="331" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="331" spans="1:14">
       <c r="A331" t="s">
         <v>14</v>
       </c>
@@ -30326,7 +30302,7 @@
         <v>5066</v>
       </c>
     </row>
-    <row r="332" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="332" spans="1:14">
       <c r="A332" t="s">
         <v>17</v>
       </c>
@@ -30370,7 +30346,7 @@
         <v>5067</v>
       </c>
     </row>
-    <row r="333" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="333" spans="1:14">
       <c r="A333" t="s">
         <v>17</v>
       </c>
@@ -30414,7 +30390,7 @@
         <v>5068</v>
       </c>
     </row>
-    <row r="334" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="334" spans="1:14">
       <c r="A334" t="s">
         <v>15</v>
       </c>
@@ -30458,7 +30434,7 @@
         <v>5069</v>
       </c>
     </row>
-    <row r="335" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="335" spans="1:14">
       <c r="A335" t="s">
         <v>14</v>
       </c>
@@ -30502,7 +30478,7 @@
         <v>5070</v>
       </c>
     </row>
-    <row r="336" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="336" spans="1:14">
       <c r="A336" t="s">
         <v>14</v>
       </c>
@@ -30546,7 +30522,7 @@
         <v>5071</v>
       </c>
     </row>
-    <row r="337" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="337" spans="1:14">
       <c r="A337" t="s">
         <v>14</v>
       </c>
@@ -30590,7 +30566,7 @@
         <v>5072</v>
       </c>
     </row>
-    <row r="338" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="338" spans="1:14">
       <c r="A338" t="s">
         <v>20</v>
       </c>
@@ -30634,7 +30610,7 @@
         <v>5073</v>
       </c>
     </row>
-    <row r="339" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="339" spans="1:14">
       <c r="A339" t="s">
         <v>14</v>
       </c>
@@ -30678,7 +30654,7 @@
         <v>5074</v>
       </c>
     </row>
-    <row r="340" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="340" spans="1:14">
       <c r="A340" t="s">
         <v>15</v>
       </c>
@@ -30722,7 +30698,7 @@
         <v>5075</v>
       </c>
     </row>
-    <row r="341" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="341" spans="1:14">
       <c r="A341" t="s">
         <v>14</v>
       </c>
@@ -30766,7 +30742,7 @@
         <v>5076</v>
       </c>
     </row>
-    <row r="342" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="342" spans="1:14">
       <c r="A342" t="s">
         <v>18</v>
       </c>
@@ -30810,7 +30786,7 @@
         <v>5077</v>
       </c>
     </row>
-    <row r="343" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="343" spans="1:14">
       <c r="A343" t="s">
         <v>18</v>
       </c>
@@ -30854,7 +30830,7 @@
         <v>5078</v>
       </c>
     </row>
-    <row r="344" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="344" spans="1:14">
       <c r="A344" t="s">
         <v>14</v>
       </c>
@@ -30898,7 +30874,7 @@
         <v>5079</v>
       </c>
     </row>
-    <row r="345" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="345" spans="1:14">
       <c r="A345" t="s">
         <v>14</v>
       </c>
@@ -30942,7 +30918,7 @@
         <v>5080</v>
       </c>
     </row>
-    <row r="346" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="346" spans="1:14">
       <c r="A346" t="s">
         <v>18</v>
       </c>
@@ -30986,7 +30962,7 @@
         <v>5081</v>
       </c>
     </row>
-    <row r="347" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="347" spans="1:14">
       <c r="A347" t="s">
         <v>14</v>
       </c>
@@ -31030,7 +31006,7 @@
         <v>5082</v>
       </c>
     </row>
-    <row r="348" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="348" spans="1:14">
       <c r="A348" t="s">
         <v>15</v>
       </c>
@@ -31074,7 +31050,7 @@
         <v>5083</v>
       </c>
     </row>
-    <row r="349" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="349" spans="1:14">
       <c r="A349" t="s">
         <v>14</v>
       </c>
@@ -31118,7 +31094,7 @@
         <v>5084</v>
       </c>
     </row>
-    <row r="350" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="350" spans="1:14">
       <c r="A350" t="s">
         <v>18</v>
       </c>
@@ -31162,7 +31138,7 @@
         <v>5085</v>
       </c>
     </row>
-    <row r="351" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="351" spans="1:14">
       <c r="A351" t="s">
         <v>14</v>
       </c>
@@ -31206,7 +31182,7 @@
         <v>5086</v>
       </c>
     </row>
-    <row r="352" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="352" spans="1:14">
       <c r="A352" t="s">
         <v>14</v>
       </c>
@@ -31250,7 +31226,7 @@
         <v>5087</v>
       </c>
     </row>
-    <row r="353" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="353" spans="1:14">
       <c r="A353" t="s">
         <v>19</v>
       </c>
@@ -31294,7 +31270,7 @@
         <v>5088</v>
       </c>
     </row>
-    <row r="354" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="354" spans="1:14">
       <c r="A354" t="s">
         <v>16</v>
       </c>
@@ -31338,7 +31314,7 @@
         <v>5089</v>
       </c>
     </row>
-    <row r="355" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="355" spans="1:14">
       <c r="A355" t="s">
         <v>14</v>
       </c>
@@ -31382,7 +31358,7 @@
         <v>5090</v>
       </c>
     </row>
-    <row r="356" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="356" spans="1:14">
       <c r="A356" t="s">
         <v>14</v>
       </c>
@@ -31426,7 +31402,7 @@
         <v>5091</v>
       </c>
     </row>
-    <row r="357" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="357" spans="1:14">
       <c r="A357" t="s">
         <v>18</v>
       </c>
@@ -31470,7 +31446,7 @@
         <v>5092</v>
       </c>
     </row>
-    <row r="358" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="358" spans="1:14">
       <c r="A358" t="s">
         <v>14</v>
       </c>
@@ -31514,7 +31490,7 @@
         <v>5093</v>
       </c>
     </row>
-    <row r="359" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="359" spans="1:14">
       <c r="A359" t="s">
         <v>14</v>
       </c>
@@ -31558,7 +31534,7 @@
         <v>5094</v>
       </c>
     </row>
-    <row r="360" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="360" spans="1:14">
       <c r="A360" t="s">
         <v>18</v>
       </c>
@@ -31602,7 +31578,7 @@
         <v>5095</v>
       </c>
     </row>
-    <row r="361" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="361" spans="1:14">
       <c r="A361" t="s">
         <v>15</v>
       </c>
@@ -31646,7 +31622,7 @@
         <v>5096</v>
       </c>
     </row>
-    <row r="362" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="362" spans="1:14">
       <c r="A362" t="s">
         <v>18</v>
       </c>
@@ -31690,7 +31666,7 @@
         <v>5097</v>
       </c>
     </row>
-    <row r="363" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="363" spans="1:14">
       <c r="A363" t="s">
         <v>19</v>
       </c>
@@ -31734,7 +31710,7 @@
         <v>5098</v>
       </c>
     </row>
-    <row r="364" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="364" spans="1:14">
       <c r="A364" t="s">
         <v>14</v>
       </c>
@@ -31778,7 +31754,7 @@
         <v>5099</v>
       </c>
     </row>
-    <row r="365" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="365" spans="1:14">
       <c r="A365" t="s">
         <v>18</v>
       </c>
@@ -31822,7 +31798,7 @@
         <v>5100</v>
       </c>
     </row>
-    <row r="366" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="366" spans="1:14">
       <c r="A366" t="s">
         <v>16</v>
       </c>
@@ -31866,7 +31842,7 @@
         <v>5101</v>
       </c>
     </row>
-    <row r="367" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="367" spans="1:14">
       <c r="A367" t="s">
         <v>14</v>
       </c>
@@ -31910,7 +31886,7 @@
         <v>5102</v>
       </c>
     </row>
-    <row r="368" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="368" spans="1:14">
       <c r="A368" t="s">
         <v>14</v>
       </c>
@@ -31954,7 +31930,7 @@
         <v>5103</v>
       </c>
     </row>
-    <row r="369" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="369" spans="1:14">
       <c r="A369" t="s">
         <v>14</v>
       </c>
@@ -31998,7 +31974,7 @@
         <v>5104</v>
       </c>
     </row>
-    <row r="370" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="370" spans="1:14">
       <c r="A370" t="s">
         <v>14</v>
       </c>
@@ -32042,7 +32018,7 @@
         <v>5105</v>
       </c>
     </row>
-    <row r="371" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="371" spans="1:14">
       <c r="A371" t="s">
         <v>14</v>
       </c>
@@ -32086,7 +32062,7 @@
         <v>5106</v>
       </c>
     </row>
-    <row r="372" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="372" spans="1:14">
       <c r="A372" t="s">
         <v>14</v>
       </c>
@@ -32130,7 +32106,7 @@
         <v>5107</v>
       </c>
     </row>
-    <row r="373" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="373" spans="1:14">
       <c r="A373" t="s">
         <v>14</v>
       </c>
@@ -32174,7 +32150,7 @@
         <v>5108</v>
       </c>
     </row>
-    <row r="374" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="374" spans="1:14">
       <c r="A374" t="s">
         <v>17</v>
       </c>
@@ -32218,7 +32194,7 @@
         <v>5109</v>
       </c>
     </row>
-    <row r="375" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="375" spans="1:14">
       <c r="A375" t="s">
         <v>14</v>
       </c>
@@ -32262,7 +32238,7 @@
         <v>5110</v>
       </c>
     </row>
-    <row r="376" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="376" spans="1:14">
       <c r="A376" t="s">
         <v>20</v>
       </c>
@@ -32306,7 +32282,7 @@
         <v>5111</v>
       </c>
     </row>
-    <row r="377" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="377" spans="1:14">
       <c r="A377" t="s">
         <v>18</v>
       </c>
@@ -32350,7 +32326,7 @@
         <v>5112</v>
       </c>
     </row>
-    <row r="378" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="378" spans="1:14">
       <c r="A378" t="s">
         <v>17</v>
       </c>
@@ -32394,7 +32370,7 @@
         <v>5113</v>
       </c>
     </row>
-    <row r="379" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="379" spans="1:14">
       <c r="A379" t="s">
         <v>14</v>
       </c>
@@ -32438,7 +32414,7 @@
         <v>5114</v>
       </c>
     </row>
-    <row r="380" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="380" spans="1:14">
       <c r="A380" t="s">
         <v>16</v>
       </c>
@@ -32482,7 +32458,7 @@
         <v>5115</v>
       </c>
     </row>
-    <row r="381" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="381" spans="1:14">
       <c r="A381" t="s">
         <v>17</v>
       </c>
@@ -32526,7 +32502,7 @@
         <v>5116</v>
       </c>
     </row>
-    <row r="382" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="382" spans="1:14">
       <c r="A382" t="s">
         <v>14</v>
       </c>
@@ -32570,7 +32546,7 @@
         <v>5117</v>
       </c>
     </row>
-    <row r="383" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="383" spans="1:14">
       <c r="A383" t="s">
         <v>14</v>
       </c>
@@ -32614,7 +32590,7 @@
         <v>5118</v>
       </c>
     </row>
-    <row r="384" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="384" spans="1:14">
       <c r="A384" t="s">
         <v>18</v>
       </c>
@@ -32658,7 +32634,7 @@
         <v>5119</v>
       </c>
     </row>
-    <row r="385" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="385" spans="1:14">
       <c r="A385" t="s">
         <v>18</v>
       </c>
@@ -32702,7 +32678,7 @@
         <v>5120</v>
       </c>
     </row>
-    <row r="386" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="386" spans="1:14">
       <c r="A386" t="s">
         <v>20</v>
       </c>
@@ -32746,7 +32722,7 @@
         <v>5121</v>
       </c>
     </row>
-    <row r="387" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="387" spans="1:14">
       <c r="A387" t="s">
         <v>14</v>
       </c>
@@ -32790,7 +32766,7 @@
         <v>5122</v>
       </c>
     </row>
-    <row r="388" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="388" spans="1:14">
       <c r="A388" t="s">
         <v>18</v>
       </c>
@@ -32834,7 +32810,7 @@
         <v>5123</v>
       </c>
     </row>
-    <row r="389" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="389" spans="1:14">
       <c r="A389" t="s">
         <v>18</v>
       </c>
@@ -32878,7 +32854,7 @@
         <v>5124</v>
       </c>
     </row>
-    <row r="390" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="390" spans="1:14">
       <c r="A390" t="s">
         <v>14</v>
       </c>
@@ -32922,7 +32898,7 @@
         <v>5125</v>
       </c>
     </row>
-    <row r="391" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="391" spans="1:14">
       <c r="A391" t="s">
         <v>19</v>
       </c>
@@ -32966,7 +32942,7 @@
         <v>5126</v>
       </c>
     </row>
-    <row r="392" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="392" spans="1:14">
       <c r="A392" t="s">
         <v>14</v>
       </c>
@@ -33010,7 +32986,7 @@
         <v>5127</v>
       </c>
     </row>
-    <row r="393" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="393" spans="1:14">
       <c r="A393" t="s">
         <v>18</v>
       </c>
@@ -33054,7 +33030,7 @@
         <v>5128</v>
       </c>
     </row>
-    <row r="394" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="394" spans="1:14">
       <c r="A394" t="s">
         <v>19</v>
       </c>

</xml_diff>